<commit_message>
🔒 [FULL] Daily chip data 2026-09-01 22:59
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -35,6 +35,7 @@
     <numFmt numFmtId="174" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="175" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="176" formatCode="#,##0.00;-#,##0.00"/>
+    <numFmt numFmtId="177" formatCode="0.0%&quot; 市-709億 &quot;&quot;(昨11/5d18)&quot;"/>
   </numFmts>
   <fonts count="50">
     <font>
@@ -581,7 +582,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="242">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1141,6 +1142,9 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2288,7 +2292,7 @@
         <v>10</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
@@ -2300,25 +2304,25 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="n">
+        <v>3239</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="J26" s="18" t="n">
+      <c r="L26" s="18" t="n">
         <v>1871</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>竹科主力分點</t>
-        </is>
-      </c>
-      <c r="L26" s="18" t="n">
-        <v>1292</v>
       </c>
       <c r="M26" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>13312</v>
+        <v>15707</v>
       </c>
     </row>
     <row r="27">
@@ -2394,7 +2398,7 @@
         </is>
       </c>
       <c r="G30" s="208" t="n">
-        <v>-23.49664</v>
+        <v>-23.14886</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2411,8 +2415,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="210" t="n">
-        <v>0.2096115874434546</v>
+      <c r="G31" s="241" t="n">
+        <v>0.2093086161180469</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2495,7 +2499,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>35.4%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2523,11 +2527,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1479730</v>
+        <v>1485604</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2539,7 +2543,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>234024</v>
+        <v>234593</v>
       </c>
       <c r="I38" s="212" t="n">
         <v>0.0271</v>
@@ -2683,22 +2687,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>巨人傑</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>巨人傑 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>3 檔</t>
+          <t>5 檔</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2714,7 @@
       </c>
       <c r="C47" s="40" t="inlineStr">
         <is>
-          <t>布哥/n_nchang</t>
+          <t>巨人傑</t>
         </is>
       </c>
       <c r="D47" s="40" t="inlineStr">
@@ -2720,7 +2724,7 @@
       </c>
       <c r="E47" s="40" t="inlineStr">
         <is>
-          <t>布哥/n_nchang 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>巨人傑 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" s="40" t="inlineStr">
@@ -2737,7 +2741,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>布哥/n_nchang</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2747,7 +2751,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>布哥/n_nchang 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2764,7 +2768,7 @@
       </c>
       <c r="C49" s="40" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D49" s="40" t="inlineStr">
@@ -2774,7 +2778,7 @@
       </c>
       <c r="E49" s="40" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" s="40" t="inlineStr">
@@ -3078,7 +3082,7 @@
         </is>
       </c>
       <c r="C64" s="33" t="n">
-        <v>1437897</v>
+        <v>1443898</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3105,7 +3109,7 @@
         <v>94068</v>
       </c>
       <c r="J64" s="213" t="n">
-        <v>0.2265536339678389</v>
+        <v>0.2256120673385749</v>
       </c>
     </row>
     <row r="65">
@@ -17562,10 +17566,10 @@
         </is>
       </c>
       <c r="E189" s="133" t="n">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="F189" s="133" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G189" s="133" t="n">
         <v>28712</v>
@@ -17577,12 +17581,12 @@
         <v>19306</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>944.46</v>
+        <v>969.99</v>
       </c>
       <c r="K189" s="134" t="n">
-        <v>959.85</v>
-      </c>
-      <c r="L189" s="237">
+        <v>969.74</v>
+      </c>
+      <c r="L189" s="236">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -17597,7 +17601,7 @@
         </is>
       </c>
       <c r="E190" s="133" t="n">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F190" s="133" t="n">
         <v>3</v>
@@ -17612,7 +17616,7 @@
         <v>19547</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>1185.88</v>
+        <v>1222.26</v>
       </c>
       <c r="K190" s="134" t="n">
         <v>1251.67</v>
@@ -17635,7 +17639,7 @@
         <v>60</v>
       </c>
       <c r="F191" s="133" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G191" s="133" t="n">
         <v>8188</v>
@@ -17650,9 +17654,9 @@
         <v>1364.62</v>
       </c>
       <c r="K191" s="134" t="n">
-        <v>1287.14</v>
-      </c>
-      <c r="L191" s="236">
+        <v>1386.15</v>
+      </c>
+      <c r="L191" s="237">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -17702,10 +17706,10 @@
         </is>
       </c>
       <c r="E193" s="133" t="n">
-        <v>164</v>
+        <v>87</v>
       </c>
       <c r="F193" s="133" t="n">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="G193" s="133" t="n">
         <v>3867</v>
@@ -17717,12 +17721,12 @@
         <v>2029</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>235.79</v>
+        <v>444.47</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>238.74</v>
-      </c>
-      <c r="L193" s="237">
+        <v>353.52</v>
+      </c>
+      <c r="L193" s="236">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -17772,10 +17776,10 @@
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>56</v>
+        <v>211</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="G195" s="133" t="n">
         <v>2893</v>
@@ -17787,12 +17791,12 @@
         <v>1662</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>516.59</v>
+        <v>137.1</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>512.92</v>
-      </c>
-      <c r="L195" s="236">
+        <v>236.73</v>
+      </c>
+      <c r="L195" s="237">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -17838,31 +17842,31 @@
       <c r="C197" s="135" t="n"/>
       <c r="D197" s="132" t="inlineStr">
         <is>
-          <t>金居(8358)</t>
+          <t>晶豪科(3006)</t>
         </is>
       </c>
       <c r="E197" s="133" t="n">
-        <v>40</v>
+        <v>87</v>
       </c>
       <c r="F197" s="133" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G197" s="133" t="n">
-        <v>2096</v>
+        <v>2423</v>
       </c>
       <c r="H197" s="133" t="n">
-        <v>490</v>
+        <v>28</v>
       </c>
       <c r="I197" s="133" t="n">
-        <v>1606</v>
+        <v>2395</v>
       </c>
       <c r="J197" s="134" t="n">
-        <v>523.9</v>
+        <v>278.51</v>
       </c>
       <c r="K197" s="134" t="n">
-        <v>544.89</v>
-      </c>
-      <c r="L197" s="237">
+        <v>278</v>
+      </c>
+      <c r="L197" s="236">
         <f>F197*(K197-J197)</f>
         <v/>
       </c>
@@ -17873,31 +17877,31 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>頎邦(6147)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>2072</v>
+        <v>2096</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>440</v>
+        <v>490</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>1632</v>
+        <v>1606</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>183.37</v>
+        <v>523.9</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>183.25</v>
-      </c>
-      <c r="L198" s="236">
+        <v>544.89</v>
+      </c>
+      <c r="L198" s="237">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -28504,7 +28508,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-01 21:38 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-01 22:59 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-02 01:42
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="16">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -36,6 +36,8 @@
     <numFmt numFmtId="175" formatCode="0&quot;%&quot;"/>
     <numFmt numFmtId="176" formatCode="#,##0.00;-#,##0.00"/>
     <numFmt numFmtId="177" formatCode="0.0%&quot; 市-709億 &quot;&quot;(昨11/5d18)&quot;"/>
+    <numFmt numFmtId="178" formatCode="0&quot; 檔 +64億 &quot;&quot;(昨15/5d11)&quot;"/>
+    <numFmt numFmtId="179" formatCode="0.0%&quot; 市-704億 &quot;&quot;(昨11/5d18)&quot;"/>
   </numFmts>
   <fonts count="50">
     <font>
@@ -582,7 +584,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1145,6 +1147,12 @@
     <xf numFmtId="177" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="178" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1230,12 +1238,12 @@
     <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 63.4%
-  • 領頭金額 78,702 萬
-  • 合計淨買 124,157 萬
+領頭大戶「陳族元」獨佔比 63.6%
+  • 領頭金額 79,367 萬
+  • 合計淨買 124,822 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 63%,
+實質 1 人下注佔 64%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1256,9 +1264,9 @@
     <comment ref="D20" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 53.6%
+領頭大戶「張濬安(航海王)」獨佔比 54.3%
   • 領頭金額 24,904 萬
-  • 合計淨買 46,428 萬
+  • 合計淨買 45,905 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 54%,
@@ -1786,33 +1794,33 @@
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>26403</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>張濬安</t>
         </is>
       </c>
-      <c r="H16" s="17" t="n">
+      <c r="J16" s="18" t="n">
         <v>21508</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>陳律師</t>
         </is>
       </c>
-      <c r="J16" s="18" t="n">
+      <c r="L16" s="18" t="n">
         <v>21175</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="L16" s="18" t="n">
-        <v>19716</v>
       </c>
       <c r="M16" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>152902</v>
+        <v>159590</v>
       </c>
     </row>
     <row r="17">
@@ -1841,7 +1849,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>78703</v>
+        <v>79368</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1863,7 +1871,7 @@
         <v>7</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>124158</v>
+        <v>124823</v>
       </c>
     </row>
     <row r="18">
@@ -1892,7 +1900,7 @@
         </is>
       </c>
       <c r="H18" s="17" t="n">
-        <v>13887</v>
+        <v>13145</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1914,7 +1922,7 @@
         <v>10</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>78294</v>
+        <v>77551</v>
       </c>
     </row>
     <row r="19">
@@ -1986,7 +1994,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2010,13 +2018,13 @@
         </is>
       </c>
       <c r="L20" s="18" t="n">
-        <v>4004</v>
+        <v>3481</v>
       </c>
       <c r="M20" s="19" t="n">
         <v>8</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>46428</v>
+        <v>45905</v>
       </c>
     </row>
     <row r="21">
@@ -2041,33 +2049,33 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
+          <t>強森</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="n">
+        <v>6655</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="n">
+        <v>6323</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H21" s="17" t="n">
-        <v>7366</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>強森</t>
-        </is>
-      </c>
-      <c r="J21" s="18" t="n">
-        <v>6655</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>張濬安</t>
-        </is>
-      </c>
       <c r="L21" s="18" t="n">
-        <v>6323</v>
+        <v>6188</v>
       </c>
       <c r="M21" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>34034</v>
+        <v>32855</v>
       </c>
     </row>
     <row r="22">
@@ -2112,13 +2120,13 @@
         </is>
       </c>
       <c r="L22" s="18" t="n">
-        <v>4993</v>
+        <v>4908</v>
       </c>
       <c r="M22" s="19" t="n">
         <v>10</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>32312</v>
+        <v>32227</v>
       </c>
     </row>
     <row r="23">
@@ -2198,7 +2206,7 @@
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>9943</v>
+        <v>8801</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2220,7 +2228,7 @@
         <v>7</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>28819</v>
+        <v>27677</v>
       </c>
     </row>
     <row r="25">
@@ -2238,10 +2246,10 @@
         </is>
       </c>
       <c r="E25" s="14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
@@ -2268,10 +2276,10 @@
         <v>1491</v>
       </c>
       <c r="M25" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N25" s="17" t="n">
-        <v>20948</v>
+        <v>21402</v>
       </c>
     </row>
     <row r="26">
@@ -2308,7 +2316,7 @@
         </is>
       </c>
       <c r="J26" s="18" t="n">
-        <v>3239</v>
+        <v>3291</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2322,7 +2330,7 @@
         <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>15707</v>
+        <v>15758</v>
       </c>
     </row>
     <row r="27">
@@ -2351,7 +2359,7 @@
         </is>
       </c>
       <c r="H27" s="17" t="n">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2373,7 +2381,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>2601</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2398,7 +2406,7 @@
         </is>
       </c>
       <c r="G30" s="208" t="n">
-        <v>-23.14886</v>
+        <v>-18.87241</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2407,7 +2415,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C31" s="209" t="n">
+      <c r="C31" s="242" t="n">
         <v>12</v>
       </c>
       <c r="F31" s="22" t="inlineStr">
@@ -2415,8 +2423,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="241" t="n">
-        <v>0.2093086161180469</v>
+      <c r="G31" s="243" t="n">
+        <v>0.2093965494893468</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2527,11 +2535,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1485604</v>
+        <v>1489239</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2543,7 +2551,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>234593</v>
+        <v>234608</v>
       </c>
       <c r="I38" s="212" t="n">
         <v>0.0271</v>
@@ -2692,17 +2700,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>5 檔</t>
+          <t>4 檔</t>
         </is>
       </c>
     </row>
@@ -2907,11 +2915,11 @@
         <v>31</v>
       </c>
       <c r="E56" t="n">
-        <v>1341522</v>
+        <v>1344709</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>陳族元 連續 31 天加碼 3008 (累計 1,341,522 萬)</t>
+          <t>陳族元 連續 31 天加碼 3008 (累計 1,344,709 萬)</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3090,7 @@
         </is>
       </c>
       <c r="C64" s="33" t="n">
-        <v>1443898</v>
+        <v>1447590</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3090,7 +3098,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>123706</v>
+        <v>124513</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3098,7 +3106,7 @@
         </is>
       </c>
       <c r="G64" s="33" t="n">
-        <v>107986</v>
+        <v>108644</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -3109,7 +3117,7 @@
         <v>94068</v>
       </c>
       <c r="J64" s="213" t="n">
-        <v>0.2256120673385749</v>
+        <v>0.2260477669617202</v>
       </c>
     </row>
     <row r="65">
@@ -5003,7 +5011,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="70" t="inlineStr">
         <is>
-          <t>-23 億 淨買</t>
+          <t>-19 億 淨買</t>
         </is>
       </c>
     </row>
@@ -17566,27 +17574,27 @@
         </is>
       </c>
       <c r="E189" s="133" t="n">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="F189" s="133" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G189" s="133" t="n">
-        <v>28712</v>
+        <v>29518</v>
       </c>
       <c r="H189" s="133" t="n">
-        <v>9406</v>
+        <v>9516</v>
       </c>
       <c r="I189" s="133" t="n">
-        <v>19306</v>
+        <v>20002</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>969.99</v>
+        <v>971</v>
       </c>
       <c r="K189" s="134" t="n">
-        <v>969.74</v>
-      </c>
-      <c r="L189" s="236">
+        <v>971</v>
+      </c>
+      <c r="L189" s="237">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -17601,25 +17609,25 @@
         </is>
       </c>
       <c r="E190" s="133" t="n">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F190" s="133" t="n">
         <v>3</v>
       </c>
       <c r="G190" s="133" t="n">
-        <v>19923</v>
+        <v>20580</v>
       </c>
       <c r="H190" s="133" t="n">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="I190" s="133" t="n">
-        <v>19547</v>
+        <v>20212</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>1222.26</v>
+        <v>1225</v>
       </c>
       <c r="K190" s="134" t="n">
-        <v>1251.67</v>
+        <v>1225</v>
       </c>
       <c r="L190" s="237">
         <f>F190*(K190-J190)</f>
@@ -17632,29 +17640,29 @@
       <c r="C191" s="135" t="n"/>
       <c r="D191" s="132" t="inlineStr">
         <is>
-          <t>雙鴻(3324)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E191" s="133" t="n">
-        <v>60</v>
+        <v>214</v>
       </c>
       <c r="F191" s="133" t="n">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="G191" s="133" t="n">
-        <v>8188</v>
+        <v>11069</v>
       </c>
       <c r="H191" s="133" t="n">
-        <v>1802</v>
+        <v>2719</v>
       </c>
       <c r="I191" s="133" t="n">
-        <v>6386</v>
+        <v>8350</v>
       </c>
       <c r="J191" s="134" t="n">
-        <v>1364.62</v>
+        <v>517.22</v>
       </c>
       <c r="K191" s="134" t="n">
-        <v>1386.15</v>
+        <v>522.9400000000001</v>
       </c>
       <c r="L191" s="237">
         <f>F191*(K191-J191)</f>
@@ -17667,31 +17675,31 @@
       <c r="C192" s="135" t="n"/>
       <c r="D192" s="132" t="inlineStr">
         <is>
-          <t>智邦(2345)</t>
+          <t>雙鴻(3324)</t>
         </is>
       </c>
       <c r="E192" s="133" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="F192" s="133" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G192" s="133" t="n">
-        <v>4268</v>
+        <v>8250</v>
       </c>
       <c r="H192" s="133" t="n">
-        <v>25</v>
+        <v>1925</v>
       </c>
       <c r="I192" s="133" t="n">
-        <v>4243</v>
+        <v>6325</v>
       </c>
       <c r="J192" s="134" t="n">
-        <v>2246.47</v>
+        <v>1375</v>
       </c>
       <c r="K192" s="134" t="n">
-        <v>252</v>
-      </c>
-      <c r="L192" s="236">
+        <v>1375</v>
+      </c>
+      <c r="L192" s="237">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -17702,31 +17710,31 @@
       <c r="C193" s="135" t="n"/>
       <c r="D193" s="132" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E193" s="133" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F193" s="133" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G193" s="133" t="n">
-        <v>3867</v>
+        <v>4058</v>
       </c>
       <c r="H193" s="133" t="n">
-        <v>1838</v>
+        <v>3595</v>
       </c>
       <c r="I193" s="133" t="n">
-        <v>2029</v>
+        <v>463</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>444.47</v>
+        <v>527.04</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>353.52</v>
-      </c>
-      <c r="L193" s="236">
+        <v>528.6900000000001</v>
+      </c>
+      <c r="L193" s="237">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -17737,29 +17745,29 @@
       <c r="C194" s="135" t="n"/>
       <c r="D194" s="132" t="inlineStr">
         <is>
-          <t>緯穎(6669)</t>
+          <t>台虹(8039)</t>
         </is>
       </c>
       <c r="E194" s="133" t="n">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="F194" s="133" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G194" s="133" t="n">
-        <v>3825</v>
+        <v>3430</v>
       </c>
       <c r="H194" s="133" t="n">
-        <v>3271</v>
+        <v>1959</v>
       </c>
       <c r="I194" s="133" t="n">
-        <v>554</v>
+        <v>1471</v>
       </c>
       <c r="J194" s="134" t="n">
-        <v>7649.2</v>
+        <v>623.58</v>
       </c>
       <c r="K194" s="134" t="n">
-        <v>8177.75</v>
+        <v>1088.33</v>
       </c>
       <c r="L194" s="237">
         <f>F194*(K194-J194)</f>
@@ -17772,29 +17780,29 @@
       <c r="C195" s="135" t="n"/>
       <c r="D195" s="132" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>旺矽(6223)</t>
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>211</v>
+        <v>6</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="G195" s="133" t="n">
-        <v>2893</v>
+        <v>3243</v>
       </c>
       <c r="H195" s="133" t="n">
-        <v>1231</v>
+        <v>635</v>
       </c>
       <c r="I195" s="133" t="n">
-        <v>1662</v>
+        <v>2608</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>137.1</v>
+        <v>5404.33</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>236.73</v>
+        <v>6354</v>
       </c>
       <c r="L195" s="237">
         <f>F195*(K195-J195)</f>
@@ -17807,29 +17815,29 @@
       <c r="C196" s="135" t="n"/>
       <c r="D196" s="132" t="inlineStr">
         <is>
-          <t>大量(3167)</t>
+          <t>大立光(3008)</t>
         </is>
       </c>
       <c r="E196" s="133" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="F196" s="133" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G196" s="133" t="n">
-        <v>2657</v>
+        <v>3187</v>
       </c>
       <c r="H196" s="133" t="n">
-        <v>1678</v>
+        <v>208</v>
       </c>
       <c r="I196" s="133" t="n">
-        <v>979</v>
+        <v>2979</v>
       </c>
       <c r="J196" s="134" t="n">
-        <v>805.09</v>
+        <v>7966.75</v>
       </c>
       <c r="K196" s="134" t="n">
-        <v>798.86</v>
+        <v>2081</v>
       </c>
       <c r="L196" s="236">
         <f>F196*(K196-J196)</f>
@@ -17846,27 +17854,27 @@
         </is>
       </c>
       <c r="E197" s="133" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F197" s="133" t="n">
         <v>1</v>
       </c>
       <c r="G197" s="133" t="n">
-        <v>2423</v>
+        <v>2475</v>
       </c>
       <c r="H197" s="133" t="n">
         <v>28</v>
       </c>
       <c r="I197" s="133" t="n">
-        <v>2395</v>
+        <v>2447</v>
       </c>
       <c r="J197" s="134" t="n">
-        <v>278.51</v>
+        <v>278.04</v>
       </c>
       <c r="K197" s="134" t="n">
-        <v>278</v>
-      </c>
-      <c r="L197" s="236">
+        <v>282</v>
+      </c>
+      <c r="L197" s="237">
         <f>F197*(K197-J197)</f>
         <v/>
       </c>
@@ -17877,29 +17885,29 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>金居(8358)</t>
+          <t>聯亞(3081)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>2096</v>
+        <v>2470</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>490</v>
+        <v>393</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>1606</v>
+        <v>2077</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>523.9</v>
+        <v>3528.29</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>544.89</v>
+        <v>3926</v>
       </c>
       <c r="L198" s="237">
         <f>F198*(K198-J198)</f>
@@ -28508,7 +28516,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-01 22:59 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 01:42 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-02 02:15
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -1238,12 +1238,12 @@
     <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 63.6%
-  • 領頭金額 79,367 萬
-  • 合計淨買 124,822 萬
+領頭大戶「陳族元」獨佔比 63.4%
+  • 領頭金額 78,702 萬
+  • 合計淨買 124,157 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 64%,
+實質 1 人下注佔 63%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1264,9 +1264,9 @@
     <comment ref="D20" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 54.3%
+領頭大戶「張濬安(航海王)」獨佔比 53.6%
   • 領頭金額 24,904 萬
-  • 合計淨買 45,905 萬
+  • 合計淨買 46,428 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 54%,
@@ -1794,33 +1794,33 @@
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>21508</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>陳律師</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>21175</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H16" s="17" t="n">
-        <v>26403</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>張濬安</t>
-        </is>
-      </c>
-      <c r="J16" s="18" t="n">
-        <v>21508</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>陳律師</t>
-        </is>
-      </c>
       <c r="L16" s="18" t="n">
-        <v>21175</v>
+        <v>19716</v>
       </c>
       <c r="M16" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>159590</v>
+        <v>152902</v>
       </c>
     </row>
     <row r="17">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>79368</v>
+        <v>78703</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>7</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>124823</v>
+        <v>124158</v>
       </c>
     </row>
     <row r="18">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="H18" s="17" t="n">
-        <v>13145</v>
+        <v>13887</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
         <v>10</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>77551</v>
+        <v>78294</v>
       </c>
     </row>
     <row r="19">
@@ -1994,7 +1994,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2018,13 +2018,13 @@
         </is>
       </c>
       <c r="L20" s="18" t="n">
-        <v>3481</v>
+        <v>4004</v>
       </c>
       <c r="M20" s="19" t="n">
         <v>8</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>45905</v>
+        <v>46428</v>
       </c>
     </row>
     <row r="21">
@@ -2049,33 +2049,33 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="n">
+        <v>7366</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H21" s="17" t="n">
+      <c r="J21" s="18" t="n">
         <v>6655</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>張濬安</t>
         </is>
       </c>
-      <c r="J21" s="18" t="n">
+      <c r="L21" s="18" t="n">
         <v>6323</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="L21" s="18" t="n">
-        <v>6188</v>
       </c>
       <c r="M21" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>32855</v>
+        <v>34034</v>
       </c>
     </row>
     <row r="22">
@@ -2120,13 +2120,13 @@
         </is>
       </c>
       <c r="L22" s="18" t="n">
-        <v>4908</v>
+        <v>4993</v>
       </c>
       <c r="M22" s="19" t="n">
         <v>10</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>32227</v>
+        <v>32312</v>
       </c>
     </row>
     <row r="23">
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>8801</v>
+        <v>9943</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         <v>7</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>27677</v>
+        <v>28819</v>
       </c>
     </row>
     <row r="25">
@@ -2246,10 +2246,10 @@
         </is>
       </c>
       <c r="E25" s="14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
@@ -2276,10 +2276,10 @@
         <v>1491</v>
       </c>
       <c r="M25" s="19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N25" s="17" t="n">
-        <v>21402</v>
+        <v>20948</v>
       </c>
     </row>
     <row r="26">
@@ -2300,7 +2300,7 @@
         <v>10</v>
       </c>
       <c r="F26" s="15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
@@ -2312,25 +2312,25 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>強森</t>
         </is>
       </c>
       <c r="J26" s="18" t="n">
-        <v>3291</v>
+        <v>1871</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>強森</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="L26" s="18" t="n">
-        <v>1871</v>
+        <v>1292</v>
       </c>
       <c r="M26" s="19" t="n">
         <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>15758</v>
+        <v>13312</v>
       </c>
     </row>
     <row r="27">
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="H27" s="17" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>2600</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2406,7 +2406,7 @@
         </is>
       </c>
       <c r="G30" s="208" t="n">
-        <v>-18.87241</v>
+        <v>-23.49664</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2415,7 +2415,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C31" s="242" t="n">
+      <c r="C31" s="209" t="n">
         <v>12</v>
       </c>
       <c r="F31" s="22" t="inlineStr">
@@ -2423,8 +2423,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="243" t="n">
-        <v>0.2093965494893468</v>
+      <c r="G31" s="210" t="n">
+        <v>0.2092273806982912</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>35.4%</t>
+          <t>35.5%</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2535,11 +2535,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1489239</v>
+        <v>1479730</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>234608</v>
+        <v>234024</v>
       </c>
       <c r="I38" s="212" t="n">
         <v>0.0271</v>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>巨人傑</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2705,12 +2705,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>巨人傑 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>4 檔</t>
+          <t>3 檔</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="C47" s="40" t="inlineStr">
         <is>
-          <t>巨人傑</t>
+          <t>布哥/n_nchang</t>
         </is>
       </c>
       <c r="D47" s="40" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="E47" s="40" t="inlineStr">
         <is>
-          <t>巨人傑 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>布哥/n_nchang 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F47" s="40" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>布哥/n_nchang</t>
+          <t>林滄海</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>布哥/n_nchang 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>林滄海 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="C49" s="40" t="inlineStr">
         <is>
-          <t>林滄海</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D49" s="40" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E49" s="40" t="inlineStr">
         <is>
-          <t>林滄海 今日買進 3 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 3 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F49" s="40" t="inlineStr">
@@ -2915,11 +2915,11 @@
         <v>31</v>
       </c>
       <c r="E56" t="n">
-        <v>1344709</v>
+        <v>1341522</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>陳族元 連續 31 天加碼 3008 (累計 1,344,709 萬)</t>
+          <t>陳族元 連續 31 天加碼 3008 (累計 1,341,522 萬)</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3090,7 @@
         </is>
       </c>
       <c r="C64" s="33" t="n">
-        <v>1447590</v>
+        <v>1437897</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>124513</v>
+        <v>123706</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="G64" s="33" t="n">
-        <v>108644</v>
+        <v>107986</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
         <v>94068</v>
       </c>
       <c r="J64" s="213" t="n">
-        <v>0.2260477669617202</v>
+        <v>0.2265536339678389</v>
       </c>
     </row>
     <row r="65">
@@ -5011,7 +5011,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="70" t="inlineStr">
         <is>
-          <t>-19 億 淨買</t>
+          <t>-23 億 淨買</t>
         </is>
       </c>
     </row>
@@ -17580,19 +17580,19 @@
         <v>98</v>
       </c>
       <c r="G189" s="133" t="n">
-        <v>29518</v>
+        <v>28712</v>
       </c>
       <c r="H189" s="133" t="n">
-        <v>9516</v>
+        <v>9406</v>
       </c>
       <c r="I189" s="133" t="n">
-        <v>20002</v>
+        <v>19306</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>971</v>
+        <v>944.46</v>
       </c>
       <c r="K189" s="134" t="n">
-        <v>971</v>
+        <v>959.85</v>
       </c>
       <c r="L189" s="237">
         <f>F189*(K189-J189)</f>
@@ -17615,19 +17615,19 @@
         <v>3</v>
       </c>
       <c r="G190" s="133" t="n">
-        <v>20580</v>
+        <v>19923</v>
       </c>
       <c r="H190" s="133" t="n">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="I190" s="133" t="n">
-        <v>20212</v>
+        <v>19547</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>1225</v>
+        <v>1185.88</v>
       </c>
       <c r="K190" s="134" t="n">
-        <v>1225</v>
+        <v>1251.67</v>
       </c>
       <c r="L190" s="237">
         <f>F190*(K190-J190)</f>
@@ -17640,31 +17640,31 @@
       <c r="C191" s="135" t="n"/>
       <c r="D191" s="132" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>雙鴻(3324)</t>
         </is>
       </c>
       <c r="E191" s="133" t="n">
-        <v>214</v>
+        <v>60</v>
       </c>
       <c r="F191" s="133" t="n">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="G191" s="133" t="n">
-        <v>11069</v>
+        <v>8188</v>
       </c>
       <c r="H191" s="133" t="n">
-        <v>2719</v>
+        <v>1802</v>
       </c>
       <c r="I191" s="133" t="n">
-        <v>8350</v>
+        <v>6386</v>
       </c>
       <c r="J191" s="134" t="n">
-        <v>517.22</v>
+        <v>1364.62</v>
       </c>
       <c r="K191" s="134" t="n">
-        <v>522.9400000000001</v>
-      </c>
-      <c r="L191" s="237">
+        <v>1287.14</v>
+      </c>
+      <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -17675,31 +17675,31 @@
       <c r="C192" s="135" t="n"/>
       <c r="D192" s="132" t="inlineStr">
         <is>
-          <t>雙鴻(3324)</t>
+          <t>智邦(2345)</t>
         </is>
       </c>
       <c r="E192" s="133" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="F192" s="133" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G192" s="133" t="n">
-        <v>8250</v>
+        <v>4268</v>
       </c>
       <c r="H192" s="133" t="n">
-        <v>1925</v>
+        <v>25</v>
       </c>
       <c r="I192" s="133" t="n">
-        <v>6325</v>
+        <v>4243</v>
       </c>
       <c r="J192" s="134" t="n">
-        <v>1375</v>
+        <v>2246.47</v>
       </c>
       <c r="K192" s="134" t="n">
-        <v>1375</v>
-      </c>
-      <c r="L192" s="237">
+        <v>252</v>
+      </c>
+      <c r="L192" s="236">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -17710,29 +17710,29 @@
       <c r="C193" s="135" t="n"/>
       <c r="D193" s="132" t="inlineStr">
         <is>
-          <t>金居(8358)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E193" s="133" t="n">
+        <v>164</v>
+      </c>
+      <c r="F193" s="133" t="n">
         <v>77</v>
       </c>
-      <c r="F193" s="133" t="n">
-        <v>68</v>
-      </c>
       <c r="G193" s="133" t="n">
-        <v>4058</v>
+        <v>3867</v>
       </c>
       <c r="H193" s="133" t="n">
-        <v>3595</v>
+        <v>1838</v>
       </c>
       <c r="I193" s="133" t="n">
-        <v>463</v>
+        <v>2029</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>527.04</v>
+        <v>235.79</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>528.6900000000001</v>
+        <v>238.74</v>
       </c>
       <c r="L193" s="237">
         <f>F193*(K193-J193)</f>
@@ -17745,29 +17745,29 @@
       <c r="C194" s="135" t="n"/>
       <c r="D194" s="132" t="inlineStr">
         <is>
-          <t>台虹(8039)</t>
+          <t>緯穎(6669)</t>
         </is>
       </c>
       <c r="E194" s="133" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="F194" s="133" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G194" s="133" t="n">
-        <v>3430</v>
+        <v>3825</v>
       </c>
       <c r="H194" s="133" t="n">
-        <v>1959</v>
+        <v>3271</v>
       </c>
       <c r="I194" s="133" t="n">
-        <v>1471</v>
+        <v>554</v>
       </c>
       <c r="J194" s="134" t="n">
-        <v>623.58</v>
+        <v>7649.2</v>
       </c>
       <c r="K194" s="134" t="n">
-        <v>1088.33</v>
+        <v>8177.75</v>
       </c>
       <c r="L194" s="237">
         <f>F194*(K194-J194)</f>
@@ -17780,31 +17780,31 @@
       <c r="C195" s="135" t="n"/>
       <c r="D195" s="132" t="inlineStr">
         <is>
-          <t>旺矽(6223)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="G195" s="133" t="n">
-        <v>3243</v>
+        <v>2893</v>
       </c>
       <c r="H195" s="133" t="n">
-        <v>635</v>
+        <v>1231</v>
       </c>
       <c r="I195" s="133" t="n">
-        <v>2608</v>
+        <v>1662</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>5404.33</v>
+        <v>516.59</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>6354</v>
-      </c>
-      <c r="L195" s="237">
+        <v>512.92</v>
+      </c>
+      <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -17815,29 +17815,29 @@
       <c r="C196" s="135" t="n"/>
       <c r="D196" s="132" t="inlineStr">
         <is>
-          <t>大立光(3008)</t>
+          <t>大量(3167)</t>
         </is>
       </c>
       <c r="E196" s="133" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="F196" s="133" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="G196" s="133" t="n">
-        <v>3187</v>
+        <v>2657</v>
       </c>
       <c r="H196" s="133" t="n">
-        <v>208</v>
+        <v>1678</v>
       </c>
       <c r="I196" s="133" t="n">
-        <v>2979</v>
+        <v>979</v>
       </c>
       <c r="J196" s="134" t="n">
-        <v>7966.75</v>
+        <v>805.09</v>
       </c>
       <c r="K196" s="134" t="n">
-        <v>2081</v>
+        <v>798.86</v>
       </c>
       <c r="L196" s="236">
         <f>F196*(K196-J196)</f>
@@ -17850,29 +17850,29 @@
       <c r="C197" s="135" t="n"/>
       <c r="D197" s="132" t="inlineStr">
         <is>
-          <t>晶豪科(3006)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E197" s="133" t="n">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="F197" s="133" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G197" s="133" t="n">
-        <v>2475</v>
+        <v>2096</v>
       </c>
       <c r="H197" s="133" t="n">
-        <v>28</v>
+        <v>490</v>
       </c>
       <c r="I197" s="133" t="n">
-        <v>2447</v>
+        <v>1606</v>
       </c>
       <c r="J197" s="134" t="n">
-        <v>278.04</v>
+        <v>523.9</v>
       </c>
       <c r="K197" s="134" t="n">
-        <v>282</v>
+        <v>544.89</v>
       </c>
       <c r="L197" s="237">
         <f>F197*(K197-J197)</f>
@@ -17885,31 +17885,31 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>聯亞(3081)</t>
+          <t>頎邦(6147)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>7</v>
+        <v>113</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>2470</v>
+        <v>2072</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>393</v>
+        <v>440</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>2077</v>
+        <v>1632</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>3528.29</v>
+        <v>183.37</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>3926</v>
-      </c>
-      <c r="L198" s="237">
+        <v>183.25</v>
+      </c>
+      <c r="L198" s="236">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -28516,7 +28516,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 01:42 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 02:15 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-02 03:12
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="G31" s="210" t="n">
-        <v>0.2092273806982912</v>
+        <v>0.2096115874434546</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -28516,7 +28516,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 02:15 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 03:12 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-02 22:56
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="20">
+  <numFmts count="22">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -43,6 +43,8 @@
     <numFmt numFmtId="181" formatCode="0&quot; 檔 +120億 &quot;&quot;(昨12/5d11)&quot;"/>
     <numFmt numFmtId="182" formatCode="0.0%&quot; 市-1611億 &quot;&quot;(昨21/5d19)&quot;"/>
     <numFmt numFmtId="183" formatCode="&quot;📅 明日預測 ↕ 中性 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
+    <numFmt numFmtId="184" formatCode="0&quot; 檔 +121億 &quot;&quot;(昨12/5d11)&quot;"/>
+    <numFmt numFmtId="185" formatCode="0.0%&quot; 市-1608億 &quot;&quot;(昨21/5d19)&quot;"/>
   </numFmts>
   <fonts count="53">
     <font>
@@ -613,7 +615,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="254">
+  <cellXfs count="256">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1206,6 +1208,12 @@
     <xf numFmtId="0" fontId="51" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="184" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1655,7 +1663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N142"/>
+  <dimension ref="B2:N141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1891,10 +1899,10 @@
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
@@ -1921,10 +1929,10 @@
         <v>40732</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>256864</v>
+        <v>268406</v>
       </c>
     </row>
     <row r="18">
@@ -2659,23 +2667,23 @@
         <v>10</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="n">
+        <v>2382</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H32" s="17" t="n">
+      <c r="J32" s="18" t="n">
         <v>1370</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="J32" s="18" t="n">
-        <v>949</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2689,7 +2697,7 @@
         <v>7</v>
       </c>
       <c r="N32" s="17" t="n">
-        <v>5185</v>
+        <v>6618</v>
       </c>
     </row>
     <row r="33">
@@ -2758,10 +2766,10 @@
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G34" s="16" t="inlineStr">
         <is>
@@ -2788,10 +2796,10 @@
         <v>132</v>
       </c>
       <c r="M34" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N34" s="17" t="n">
-        <v>1608</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2816,7 +2824,7 @@
         </is>
       </c>
       <c r="G37" s="244" t="n">
-        <v>-151.23464</v>
+        <v>-148.32073</v>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
@@ -2825,7 +2833,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C38" s="245" t="n">
+      <c r="C38" s="254" t="n">
         <v>19</v>
       </c>
       <c r="F38" s="22" t="inlineStr">
@@ -2833,8 +2841,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G38" s="246" t="n">
-        <v>0.2027315599898919</v>
+      <c r="G38" s="255" t="n">
+        <v>0.2035157242394799</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
@@ -2917,7 +2925,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2945,11 +2953,11 @@
         </is>
       </c>
       <c r="D45" s="33" t="n">
-        <v>929828</v>
+        <v>951729</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2961,7 +2969,7 @@
         </is>
       </c>
       <c r="H45" s="33" t="n">
-        <v>256864</v>
+        <v>268406</v>
       </c>
       <c r="I45" s="234" t="n">
         <v>-0.009300000000000001</v>
@@ -2981,7 +2989,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -3013,7 +3021,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -3045,7 +3053,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -3213,22 +3221,22 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 5 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>5 檔</t>
+          <t>4 檔</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3248,7 @@
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="D58" s="40" t="inlineStr">
@@ -3250,7 +3258,7 @@
       </c>
       <c r="E58" s="40" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>竹科主力分點 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F58" s="40" t="inlineStr">
@@ -3267,7 +3275,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>蔣承翰</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3277,7 +3285,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>竹科主力分點 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>蔣承翰 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3294,7 +3302,7 @@
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
-          <t>蔣承翰</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D60" s="40" t="inlineStr">
@@ -3304,7 +3312,7 @@
       </c>
       <c r="E60" s="40" t="inlineStr">
         <is>
-          <t>蔣承翰 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F60" s="40" t="inlineStr">
@@ -3648,7 +3656,7 @@
         </is>
       </c>
       <c r="C77" s="33" t="n">
-        <v>877076</v>
+        <v>900821</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3675,7 +3683,7 @@
         <v>76726</v>
       </c>
       <c r="J77" s="213" t="n">
-        <v>0.2905248472737998</v>
+        <v>0.28286672585709</v>
       </c>
     </row>
     <row r="78">
@@ -4088,7 +4096,7 @@
     <row r="90" ht="22" customHeight="1">
       <c r="B90" s="57" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260901)</t>
+          <t>▍ G. 注意股 (資料日 20260902)</t>
         </is>
       </c>
     </row>
@@ -4122,19 +4130,19 @@
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>047757</t>
+          <t>066185</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>南電中信5C購02</t>
+          <t>聯發科元大64購05</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>25.5</v>
+        <v>1.64</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -4145,19 +4153,19 @@
     <row r="93">
       <c r="B93" s="40" t="inlineStr">
         <is>
-          <t>1312</t>
+          <t>069544</t>
         </is>
       </c>
       <c r="C93" s="40" t="inlineStr">
         <is>
-          <t>國喬</t>
+          <t>立隆電元大5B購05</t>
         </is>
       </c>
       <c r="D93" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E93" s="40" t="n">
-        <v>15.65</v>
+        <v>0.14</v>
       </c>
       <c r="F93" s="40" t="inlineStr">
         <is>
@@ -4168,69 +4176,69 @@
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>2426</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>鼎元</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>1225</v>
+        <v>104.5</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>43.97</t>
+          <t>1045.00</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="40" t="inlineStr">
         <is>
-          <t>2426</t>
+          <t>2455</t>
         </is>
       </c>
       <c r="C95" s="40" t="inlineStr">
         <is>
-          <t>鼎元</t>
+          <t>全新</t>
         </is>
       </c>
       <c r="D95" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E95" s="40" t="n">
-        <v>107.5</v>
+        <v>542</v>
       </c>
       <c r="F95" s="40" t="inlineStr">
         <is>
-          <t>1075.00</t>
+          <t>132.84</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>2455</t>
+          <t>2466</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>全新</t>
+          <t>冠西電</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>524</v>
+        <v>104</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>128.43</t>
+          <t>66.24</t>
         </is>
       </c>
     </row>
@@ -4249,980 +4257,957 @@
         <v>1</v>
       </c>
       <c r="E97" s="40" t="n">
-        <v>7580</v>
+        <v>7810</v>
       </c>
       <c r="F97" s="40" t="inlineStr">
         <is>
-          <t>40.31</t>
+          <t>41.54</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>3406</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>玉晶光</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>971</v>
+        <v>1050</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>64.65</t>
+          <t>28.41</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" s="40" t="inlineStr">
         <is>
-          <t>3055</t>
+          <t>3450</t>
         </is>
       </c>
       <c r="C99" s="40" t="inlineStr">
         <is>
-          <t>蔚華科</t>
+          <t>聯鈞</t>
         </is>
       </c>
       <c r="D99" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E99" s="40" t="n">
-        <v>129.5</v>
+        <v>602</v>
       </c>
       <c r="F99" s="40" t="inlineStr">
         <is>
-          <t>-----</t>
+          <t>122.11</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>6226</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>光鼎</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>874</v>
+        <v>34.15</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>162.15</t>
+          <t>-----</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" s="40" t="inlineStr">
         <is>
-          <t>3406</t>
+          <t>6834</t>
         </is>
       </c>
       <c r="C101" s="40" t="inlineStr">
         <is>
-          <t>玉晶光</t>
+          <t>天二科技</t>
         </is>
       </c>
       <c r="D101" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E101" s="40" t="n">
-        <v>1005</v>
+        <v>92.2</v>
       </c>
       <c r="F101" s="40" t="inlineStr">
         <is>
-          <t>27.19</t>
+          <t>40.09</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>3450</t>
+          <t>6933</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>聯鈞</t>
+          <t>AMAX-KY</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>625</v>
+        <v>331</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>126.77</t>
+          <t>41.07</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="B103" s="40" t="inlineStr">
         <is>
-          <t>6209</t>
+          <t>8039</t>
         </is>
       </c>
       <c r="C103" s="40" t="inlineStr">
         <is>
-          <t>今國光</t>
+          <t>台虹</t>
         </is>
       </c>
       <c r="D103" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E103" s="40" t="n">
-        <v>81.90000000000001</v>
+        <v>313.5</v>
       </c>
       <c r="F103" s="40" t="inlineStr">
         <is>
-          <t>35.45</t>
+          <t>99.52</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>6226</t>
+          <t>8473</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>光鼎</t>
+          <t>山林水</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>34</v>
+        <v>45.95</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>-----</t>
+          <t>13.32</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" s="40" t="inlineStr">
         <is>
-          <t>6669</t>
+          <t>911608</t>
         </is>
       </c>
       <c r="C105" s="40" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>明輝-DR</t>
         </is>
       </c>
       <c r="D105" s="40" t="n">
         <v>1</v>
       </c>
       <c r="E105" s="40" t="n">
-        <v>7800</v>
+        <v>2.72</v>
       </c>
       <c r="F105" s="40" t="inlineStr">
         <is>
-          <t>25.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>6805</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>富世達</t>
-        </is>
-      </c>
-      <c r="D106" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" t="n">
-        <v>2285</v>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>48.88</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="22" customHeight="1">
-      <c r="B108" s="4" t="inlineStr">
+          <t>-----</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>▍ H. 借券賣出 Top 15 (機構級反向力量, 資料日 20260902)</t>
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="B108" s="12" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="C108" s="12" t="inlineStr">
+        <is>
+          <t>名稱</t>
+        </is>
+      </c>
+      <c r="D108" s="12" t="inlineStr">
+        <is>
+          <t>借券張數</t>
+        </is>
+      </c>
+      <c r="E108" s="12" t="inlineStr">
+        <is>
+          <t>融券張數</t>
+        </is>
+      </c>
+      <c r="F108" s="12" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+    </row>
     <row r="109">
-      <c r="B109" s="12" t="inlineStr">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>00685L</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>群益臺灣加權正2</t>
+        </is>
+      </c>
+      <c r="D109" s="33" t="n">
+        <v>30217</v>
+      </c>
+      <c r="E109" s="33" t="n">
+        <v>521</v>
+      </c>
+      <c r="F109" s="215" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="40" t="inlineStr">
+        <is>
+          <t>2887</t>
+        </is>
+      </c>
+      <c r="C110" s="40" t="inlineStr">
+        <is>
+          <t>台新新光金</t>
+        </is>
+      </c>
+      <c r="D110" s="60" t="n">
+        <v>16341</v>
+      </c>
+      <c r="E110" s="60" t="n">
+        <v>69</v>
+      </c>
+      <c r="F110" s="216" t="n">
+        <v>236.83</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>00712</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>復華富時不動產</t>
+        </is>
+      </c>
+      <c r="D111" s="33" t="n">
+        <v>7743</v>
+      </c>
+      <c r="E111" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="40" t="inlineStr">
+        <is>
+          <t>00673R</t>
+        </is>
+      </c>
+      <c r="C112" s="40" t="inlineStr">
+        <is>
+          <t>期元大S&amp;P原油反1</t>
+        </is>
+      </c>
+      <c r="D112" s="60" t="n">
+        <v>6645</v>
+      </c>
+      <c r="E112" s="60" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F112" s="216" t="n">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2883</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>凱基金</t>
+        </is>
+      </c>
+      <c r="D113" s="33" t="n">
+        <v>6239</v>
+      </c>
+      <c r="E113" s="33" t="n">
+        <v>48</v>
+      </c>
+      <c r="F113" s="215" t="n">
+        <v>129.98</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="40" t="inlineStr">
+        <is>
+          <t>00918</t>
+        </is>
+      </c>
+      <c r="C114" s="40" t="inlineStr">
+        <is>
+          <t>大華優利高填息30</t>
+        </is>
+      </c>
+      <c r="D114" s="60" t="n">
+        <v>6004</v>
+      </c>
+      <c r="E114" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2801</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>彰銀</t>
+        </is>
+      </c>
+      <c r="D115" s="33" t="n">
+        <v>4623</v>
+      </c>
+      <c r="E115" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="F115" s="215" t="n">
+        <v>420.27</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="40" t="inlineStr">
+        <is>
+          <t>3481</t>
+        </is>
+      </c>
+      <c r="C116" s="40" t="inlineStr">
+        <is>
+          <t>群創</t>
+        </is>
+      </c>
+      <c r="D116" s="60" t="n">
+        <v>4265</v>
+      </c>
+      <c r="E116" s="60" t="n">
+        <v>324</v>
+      </c>
+      <c r="F116" s="216" t="n">
+        <v>13.16</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>00919</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>群益台灣精選高息</t>
+        </is>
+      </c>
+      <c r="D117" s="33" t="n">
+        <v>4195</v>
+      </c>
+      <c r="E117" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="F117" s="215" t="n">
+        <v>599.29</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="40" t="inlineStr">
+        <is>
+          <t>1714</t>
+        </is>
+      </c>
+      <c r="C118" s="40" t="inlineStr">
+        <is>
+          <t>和桐</t>
+        </is>
+      </c>
+      <c r="D118" s="60" t="n">
+        <v>4177</v>
+      </c>
+      <c r="E118" s="60" t="n">
+        <v>104</v>
+      </c>
+      <c r="F118" s="216" t="n">
+        <v>40.16</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2327</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>國巨*</t>
+        </is>
+      </c>
+      <c r="D119" s="33" t="n">
+        <v>4078</v>
+      </c>
+      <c r="E119" s="33" t="n">
+        <v>53</v>
+      </c>
+      <c r="F119" s="215" t="n">
+        <v>76.94</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="40" t="inlineStr">
+        <is>
+          <t>2890</t>
+        </is>
+      </c>
+      <c r="C120" s="40" t="inlineStr">
+        <is>
+          <t>永豐金</t>
+        </is>
+      </c>
+      <c r="D120" s="60" t="n">
+        <v>4043</v>
+      </c>
+      <c r="E120" s="60" t="n">
+        <v>17</v>
+      </c>
+      <c r="F120" s="216" t="n">
+        <v>237.82</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="43" t="inlineStr">
+        <is>
+          <t>🔴 2002</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>中鋼</t>
+        </is>
+      </c>
+      <c r="D121" s="33" t="n">
+        <v>3921</v>
+      </c>
+      <c r="E121" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F121" s="252" t="n">
+        <v>1960.5</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="40" t="inlineStr">
+        <is>
+          <t>00403A</t>
+        </is>
+      </c>
+      <c r="C122" s="40" t="inlineStr">
+        <is>
+          <t>主動統一升級50</t>
+        </is>
+      </c>
+      <c r="D122" s="60" t="n">
+        <v>3651</v>
+      </c>
+      <c r="E122" s="60" t="n">
+        <v>165</v>
+      </c>
+      <c r="F122" s="216" t="n">
+        <v>22.13</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2880</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>華南金</t>
+        </is>
+      </c>
+      <c r="D123" s="33" t="n">
+        <v>3364</v>
+      </c>
+      <c r="E123" s="33" t="n">
+        <v>47</v>
+      </c>
+      <c r="F123" s="215" t="n">
+        <v>71.56999999999999</v>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="B125" s="62" t="inlineStr">
+        <is>
+          <t>▍ I. 未來 30 天除權息 (有效 91 檔, 已剔除過期)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="58" t="inlineStr">
+        <is>
+          <t>除權息日</t>
+        </is>
+      </c>
+      <c r="C126" s="58" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C109" s="12" t="inlineStr">
+      <c r="D126" s="58" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D109" s="12" t="inlineStr">
-        <is>
-          <t>借券張數</t>
-        </is>
-      </c>
-      <c r="E109" s="12" t="inlineStr">
-        <is>
-          <t>融券張數</t>
-        </is>
-      </c>
-      <c r="F109" s="12" t="inlineStr">
-        <is>
-          <t>ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>00685L</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>群益臺灣加權正2</t>
-        </is>
-      </c>
-      <c r="D110" s="33" t="n">
-        <v>30217</v>
-      </c>
-      <c r="E110" s="33" t="n">
-        <v>521</v>
-      </c>
-      <c r="F110" s="215" t="n">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="B111" s="40" t="inlineStr">
-        <is>
-          <t>2887</t>
-        </is>
-      </c>
-      <c r="C111" s="40" t="inlineStr">
-        <is>
-          <t>台新新光金</t>
-        </is>
-      </c>
-      <c r="D111" s="60" t="n">
-        <v>16341</v>
-      </c>
-      <c r="E111" s="60" t="n">
-        <v>69</v>
-      </c>
-      <c r="F111" s="216" t="n">
-        <v>236.83</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>00712</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>復華富時不動產</t>
-        </is>
-      </c>
-      <c r="D112" s="33" t="n">
-        <v>7743</v>
-      </c>
-      <c r="E112" s="33" t="n">
+      <c r="E126" s="58" t="inlineStr">
+        <is>
+          <t>類型</t>
+        </is>
+      </c>
+      <c r="F126" s="58" t="inlineStr">
+        <is>
+          <t>現金股利</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>00406A</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>主動中信台灣收益</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>0.138</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="40" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C128" s="40" t="inlineStr">
+        <is>
+          <t>00946</t>
+        </is>
+      </c>
+      <c r="D128" s="40" t="inlineStr">
+        <is>
+          <t>群益科技高息成長</t>
+        </is>
+      </c>
+      <c r="E128" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F128" s="40" t="n">
+        <v>0.058</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>00953B</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>群益優選非投等債</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>0.067</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="40" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C130" s="40" t="inlineStr">
+        <is>
+          <t>00985B</t>
+        </is>
+      </c>
+      <c r="D130" s="40" t="inlineStr">
+        <is>
+          <t>群益ESG投等債0-5</t>
+        </is>
+      </c>
+      <c r="E130" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F130" s="40" t="n">
+        <v>0.053</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>2464</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>盟立</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>0.471403</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="40" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C132" s="40" t="inlineStr">
+        <is>
+          <t>2845</t>
+        </is>
+      </c>
+      <c r="D132" s="40" t="inlineStr">
+        <is>
+          <t>遠東銀</t>
+        </is>
+      </c>
+      <c r="E132" s="40" t="inlineStr">
+        <is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F132" s="40" t="n">
+        <v>0.514</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>2923</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>鼎固-KY</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="B134" s="40" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C134" s="40" t="inlineStr">
+        <is>
+          <t>3013</t>
+        </is>
+      </c>
+      <c r="D134" s="40" t="inlineStr">
+        <is>
+          <t>晟銘電</t>
+        </is>
+      </c>
+      <c r="E134" s="40" t="inlineStr">
+        <is>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F134" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="B113" s="40" t="inlineStr">
-        <is>
-          <t>00673R</t>
-        </is>
-      </c>
-      <c r="C113" s="40" t="inlineStr">
-        <is>
-          <t>期元大S&amp;P原油反1</t>
-        </is>
-      </c>
-      <c r="D113" s="60" t="n">
-        <v>6645</v>
-      </c>
-      <c r="E113" s="60" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F113" s="216" t="n">
-        <v>1.33</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>2883</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>凱基金</t>
-        </is>
-      </c>
-      <c r="D114" s="33" t="n">
-        <v>6239</v>
-      </c>
-      <c r="E114" s="33" t="n">
-        <v>48</v>
-      </c>
-      <c r="F114" s="215" t="n">
-        <v>129.98</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="B115" s="40" t="inlineStr">
-        <is>
-          <t>00918</t>
-        </is>
-      </c>
-      <c r="C115" s="40" t="inlineStr">
-        <is>
-          <t>大華優利高填息30</t>
-        </is>
-      </c>
-      <c r="D115" s="60" t="n">
-        <v>6004</v>
-      </c>
-      <c r="E115" s="60" t="n">
+    </row>
+    <row r="135">
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>3346</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>麗清</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="B136" s="40" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C136" s="40" t="inlineStr">
+        <is>
+          <t>4438</t>
+        </is>
+      </c>
+      <c r="D136" s="40" t="inlineStr">
+        <is>
+          <t>廣越</t>
+        </is>
+      </c>
+      <c r="E136" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F136" s="40" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>6139</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>亞翔</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>22.996187</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="B138" s="40" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C138" s="40" t="inlineStr">
+        <is>
+          <t>6426</t>
+        </is>
+      </c>
+      <c r="D138" s="40" t="inlineStr">
+        <is>
+          <t>統新</t>
+        </is>
+      </c>
+      <c r="E138" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F138" s="40" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>20260902</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
         <v>0</v>
       </c>
-      <c r="F115" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>2801</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>彰銀</t>
-        </is>
-      </c>
-      <c r="D116" s="33" t="n">
-        <v>4623</v>
-      </c>
-      <c r="E116" s="33" t="n">
-        <v>11</v>
-      </c>
-      <c r="F116" s="215" t="n">
-        <v>420.27</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="B117" s="40" t="inlineStr">
-        <is>
-          <t>3481</t>
-        </is>
-      </c>
-      <c r="C117" s="40" t="inlineStr">
-        <is>
-          <t>群創</t>
-        </is>
-      </c>
-      <c r="D117" s="60" t="n">
-        <v>4265</v>
-      </c>
-      <c r="E117" s="60" t="n">
-        <v>324</v>
-      </c>
-      <c r="F117" s="216" t="n">
-        <v>13.16</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>00919</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>群益台灣精選高息</t>
-        </is>
-      </c>
-      <c r="D118" s="33" t="n">
-        <v>4195</v>
-      </c>
-      <c r="E118" s="33" t="n">
-        <v>7</v>
-      </c>
-      <c r="F118" s="215" t="n">
-        <v>599.29</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="B119" s="40" t="inlineStr">
-        <is>
-          <t>1714</t>
-        </is>
-      </c>
-      <c r="C119" s="40" t="inlineStr">
-        <is>
-          <t>和桐</t>
-        </is>
-      </c>
-      <c r="D119" s="60" t="n">
-        <v>4177</v>
-      </c>
-      <c r="E119" s="60" t="n">
-        <v>104</v>
-      </c>
-      <c r="F119" s="216" t="n">
-        <v>40.16</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>2327</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>國巨*</t>
-        </is>
-      </c>
-      <c r="D120" s="33" t="n">
-        <v>4078</v>
-      </c>
-      <c r="E120" s="33" t="n">
-        <v>53</v>
-      </c>
-      <c r="F120" s="215" t="n">
-        <v>76.94</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="B121" s="40" t="inlineStr">
-        <is>
-          <t>2890</t>
-        </is>
-      </c>
-      <c r="C121" s="40" t="inlineStr">
-        <is>
-          <t>永豐金</t>
-        </is>
-      </c>
-      <c r="D121" s="60" t="n">
-        <v>4043</v>
-      </c>
-      <c r="E121" s="60" t="n">
-        <v>17</v>
-      </c>
-      <c r="F121" s="216" t="n">
-        <v>237.82</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="B122" s="43" t="inlineStr">
-        <is>
-          <t>🔴 2002</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>中鋼</t>
-        </is>
-      </c>
-      <c r="D122" s="33" t="n">
-        <v>3921</v>
-      </c>
-      <c r="E122" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F122" s="252" t="n">
-        <v>1960.5</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="B123" s="40" t="inlineStr">
-        <is>
-          <t>00403A</t>
-        </is>
-      </c>
-      <c r="C123" s="40" t="inlineStr">
-        <is>
-          <t>主動統一升級50</t>
-        </is>
-      </c>
-      <c r="D123" s="60" t="n">
-        <v>3651</v>
-      </c>
-      <c r="E123" s="60" t="n">
-        <v>165</v>
-      </c>
-      <c r="F123" s="216" t="n">
-        <v>22.13</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>2880</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>華南金</t>
-        </is>
-      </c>
-      <c r="D124" s="33" t="n">
-        <v>3364</v>
-      </c>
-      <c r="E124" s="33" t="n">
-        <v>47</v>
-      </c>
-      <c r="F124" s="215" t="n">
-        <v>71.56999999999999</v>
-      </c>
-    </row>
-    <row r="126" ht="22" customHeight="1">
-      <c r="B126" s="62" t="inlineStr">
-        <is>
-          <t>▍ I. 未來 30 天除權息 (有效 84 檔, 已剔除過期)</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="B127" s="58" t="inlineStr">
-        <is>
-          <t>除權息日</t>
-        </is>
-      </c>
-      <c r="C127" s="58" t="inlineStr">
-        <is>
-          <t>代號</t>
-        </is>
-      </c>
-      <c r="D127" s="58" t="inlineStr">
-        <is>
-          <t>名稱</t>
-        </is>
-      </c>
-      <c r="E127" s="58" t="inlineStr">
-        <is>
-          <t>類型</t>
-        </is>
-      </c>
-      <c r="F127" s="58" t="inlineStr">
-        <is>
-          <t>現金股利</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="B128" t="inlineStr">
+    </row>
+    <row r="140">
+      <c r="B140" s="40" t="inlineStr">
         <is>
           <t>20260902</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>00406A</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>主動中信台灣收益</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
+      <c r="C140" s="40" t="inlineStr">
+        <is>
+          <t>6753</t>
+        </is>
+      </c>
+      <c r="D140" s="40" t="inlineStr">
+        <is>
+          <t>龍德造船</t>
+        </is>
+      </c>
+      <c r="E140" s="40" t="inlineStr">
         <is>
           <t>息</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>0.138</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="B129" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C129" s="40" t="inlineStr">
-        <is>
-          <t>00946</t>
-        </is>
-      </c>
-      <c r="D129" s="40" t="inlineStr">
-        <is>
-          <t>群益科技高息成長</t>
-        </is>
-      </c>
-      <c r="E129" s="40" t="inlineStr">
+      <c r="F140" s="40" t="n">
+        <v>1.249351</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>20260903</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>1203</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>味王</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
         <is>
           <t>息</t>
         </is>
       </c>
-      <c r="F129" s="40" t="n">
-        <v>0.058</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>00953B</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>群益優選非投等債</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F130" t="n">
-        <v>0.067</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="B131" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C131" s="40" t="inlineStr">
-        <is>
-          <t>00985B</t>
-        </is>
-      </c>
-      <c r="D131" s="40" t="inlineStr">
-        <is>
-          <t>群益ESG投等債0-5</t>
-        </is>
-      </c>
-      <c r="E131" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F131" s="40" t="n">
-        <v>0.053</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>2464</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>盟立</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>權息</t>
-        </is>
-      </c>
-      <c r="F132" t="n">
-        <v>0.471403</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="B133" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C133" s="40" t="inlineStr">
-        <is>
-          <t>2845</t>
-        </is>
-      </c>
-      <c r="D133" s="40" t="inlineStr">
-        <is>
-          <t>遠東銀</t>
-        </is>
-      </c>
-      <c r="E133" s="40" t="inlineStr">
-        <is>
-          <t>權息</t>
-        </is>
-      </c>
-      <c r="F133" s="40" t="n">
-        <v>0.514</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>2923</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>鼎固-KY</t>
-        </is>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F134" t="n">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="B135" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C135" s="40" t="inlineStr">
-        <is>
-          <t>3013</t>
-        </is>
-      </c>
-      <c r="D135" s="40" t="inlineStr">
-        <is>
-          <t>晟銘電</t>
-        </is>
-      </c>
-      <c r="E135" s="40" t="inlineStr">
-        <is>
-          <t>權</t>
-        </is>
-      </c>
-      <c r="F135" s="40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>3346</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>麗清</t>
-        </is>
-      </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F136" t="n">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="B137" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C137" s="40" t="inlineStr">
-        <is>
-          <t>4438</t>
-        </is>
-      </c>
-      <c r="D137" s="40" t="inlineStr">
-        <is>
-          <t>廣越</t>
-        </is>
-      </c>
-      <c r="E137" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F137" s="40" t="n">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>6139</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>亞翔</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F138" t="n">
-        <v>22.996187</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="B139" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C139" s="40" t="inlineStr">
-        <is>
-          <t>6426</t>
-        </is>
-      </c>
-      <c r="D139" s="40" t="inlineStr">
-        <is>
-          <t>統新</t>
-        </is>
-      </c>
-      <c r="E139" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F139" s="40" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>6669</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>緯穎</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>權</t>
-        </is>
-      </c>
-      <c r="F140" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="B141" s="40" t="inlineStr">
-        <is>
-          <t>20260902</t>
-        </is>
-      </c>
-      <c r="C141" s="40" t="inlineStr">
-        <is>
-          <t>6753</t>
-        </is>
-      </c>
-      <c r="D141" s="40" t="inlineStr">
-        <is>
-          <t>龍德造船</t>
-        </is>
-      </c>
-      <c r="E141" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F141" s="40" t="n">
-        <v>1.249351</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>20260903</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>1203</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>味王</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F142" t="n">
+      <c r="F141" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5231,9 +5216,9 @@
     <mergeCell ref="G38:I38"/>
     <mergeCell ref="B9:N9"/>
     <mergeCell ref="G37:I37"/>
+    <mergeCell ref="B107:J107"/>
     <mergeCell ref="B40:N40"/>
     <mergeCell ref="B4:N4"/>
-    <mergeCell ref="B108:J108"/>
     <mergeCell ref="B65:J65"/>
     <mergeCell ref="B7:N7"/>
     <mergeCell ref="B3:N3"/>
@@ -5242,7 +5227,6 @@
     <mergeCell ref="B51:J51"/>
     <mergeCell ref="B36:J36"/>
     <mergeCell ref="B12:N12"/>
-    <mergeCell ref="B126:J126"/>
     <mergeCell ref="B39:N39"/>
     <mergeCell ref="B11:N11"/>
     <mergeCell ref="B42:E42"/>
@@ -5251,6 +5235,7 @@
     <mergeCell ref="B14:N14"/>
     <mergeCell ref="B90:J90"/>
     <mergeCell ref="C38:D38"/>
+    <mergeCell ref="B125:J125"/>
     <mergeCell ref="B8:N8"/>
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="B13:N13"/>
@@ -5329,7 +5314,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D92:D106">
+  <conditionalFormatting sqref="D92:D105">
     <cfRule type="dataBar" priority="9">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -5338,7 +5323,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D110:D124">
+  <conditionalFormatting sqref="D109:D123">
     <cfRule type="dataBar" priority="10">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -5347,7 +5332,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F110:F124">
+  <conditionalFormatting sqref="F109:F123">
     <cfRule type="dataBar" priority="11">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
@@ -5416,7 +5401,7 @@
     <row r="9">
       <c r="C9" s="66" t="inlineStr">
         <is>
-          <t>② 聯發科 (2454) · 10 大戶</t>
+          <t>② 聯發科 (2454) · 11 大戶</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5513,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-151 億 淨買</t>
+          <t>-148 億 淨買</t>
         </is>
       </c>
     </row>
@@ -18455,29 +18440,29 @@
       </c>
       <c r="D189" s="132" t="inlineStr">
         <is>
-          <t>全新(2455)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E189" s="133" t="n">
-        <v>276</v>
+        <v>50</v>
       </c>
       <c r="F189" s="133" t="n">
-        <v>245</v>
+        <v>23</v>
       </c>
       <c r="G189" s="133" t="n">
-        <v>14958</v>
+        <v>21375</v>
       </c>
       <c r="H189" s="133" t="n">
-        <v>13291</v>
+        <v>9832</v>
       </c>
       <c r="I189" s="133" t="n">
-        <v>1667</v>
+        <v>11543</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>541.97</v>
+        <v>4275</v>
       </c>
       <c r="K189" s="134" t="n">
-        <v>542.49</v>
+        <v>4275</v>
       </c>
       <c r="L189" s="237">
         <f>F189*(K189-J189)</f>
@@ -18490,29 +18475,29 @@
       <c r="C190" s="135" t="n"/>
       <c r="D190" s="132" t="inlineStr">
         <is>
-          <t>華星光(4979)</t>
+          <t>全新(2455)</t>
         </is>
       </c>
       <c r="E190" s="133" t="n">
-        <v>90</v>
+        <v>276</v>
       </c>
       <c r="F190" s="133" t="n">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="G190" s="133" t="n">
-        <v>5539</v>
+        <v>14958</v>
       </c>
       <c r="H190" s="133" t="n">
-        <v>0</v>
+        <v>13291</v>
       </c>
       <c r="I190" s="133" t="n">
-        <v>5539</v>
+        <v>1667</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>615.4</v>
+        <v>541.97</v>
       </c>
       <c r="K190" s="134" t="n">
-        <v>0</v>
+        <v>542.49</v>
       </c>
       <c r="L190" s="237">
         <f>F190*(K190-J190)</f>
@@ -18525,29 +18510,29 @@
       <c r="C191" s="135" t="n"/>
       <c r="D191" s="132" t="inlineStr">
         <is>
-          <t>禾伸堂(3026)</t>
+          <t>華星光(4979)</t>
         </is>
       </c>
       <c r="E191" s="133" t="n">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="F191" s="133" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G191" s="133" t="n">
-        <v>4669</v>
+        <v>5539</v>
       </c>
       <c r="H191" s="133" t="n">
-        <v>1652</v>
+        <v>0</v>
       </c>
       <c r="I191" s="133" t="n">
-        <v>3017</v>
+        <v>5539</v>
       </c>
       <c r="J191" s="134" t="n">
-        <v>686.62</v>
+        <v>622.3099999999999</v>
       </c>
       <c r="K191" s="134" t="n">
-        <v>688.33</v>
+        <v>0</v>
       </c>
       <c r="L191" s="237">
         <f>F191*(K191-J191)</f>
@@ -18560,29 +18545,29 @@
       <c r="C192" s="135" t="n"/>
       <c r="D192" s="132" t="inlineStr">
         <is>
-          <t>台光電(2383)</t>
+          <t>禾伸堂(3026)</t>
         </is>
       </c>
       <c r="E192" s="133" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="F192" s="133" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G192" s="133" t="n">
-        <v>4447</v>
+        <v>4669</v>
       </c>
       <c r="H192" s="133" t="n">
-        <v>0</v>
+        <v>1652</v>
       </c>
       <c r="I192" s="133" t="n">
-        <v>4447</v>
+        <v>3017</v>
       </c>
       <c r="J192" s="134" t="n">
-        <v>5559.12</v>
+        <v>686.62</v>
       </c>
       <c r="K192" s="134" t="n">
-        <v>0</v>
+        <v>688.33</v>
       </c>
       <c r="L192" s="237">
         <f>F192*(K192-J192)</f>
@@ -18595,29 +18580,29 @@
       <c r="C193" s="135" t="n"/>
       <c r="D193" s="132" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>台光電(2383)</t>
         </is>
       </c>
       <c r="E193" s="133" t="n">
-        <v>170</v>
+        <v>8</v>
       </c>
       <c r="F193" s="133" t="n">
-        <v>143</v>
+        <v>0</v>
       </c>
       <c r="G193" s="133" t="n">
-        <v>4045</v>
+        <v>4447</v>
       </c>
       <c r="H193" s="133" t="n">
-        <v>3405</v>
+        <v>0</v>
       </c>
       <c r="I193" s="133" t="n">
-        <v>640</v>
+        <v>4447</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>237.96</v>
+        <v>5559.12</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>238.12</v>
+        <v>0</v>
       </c>
       <c r="L193" s="237">
         <f>F193*(K193-J193)</f>
@@ -18630,31 +18615,31 @@
       <c r="C194" s="135" t="n"/>
       <c r="D194" s="132" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E194" s="133" t="n">
-        <v>16</v>
+        <v>170</v>
       </c>
       <c r="F194" s="133" t="n">
-        <v>2</v>
+        <v>143</v>
       </c>
       <c r="G194" s="133" t="n">
-        <v>3933</v>
+        <v>4045</v>
       </c>
       <c r="H194" s="133" t="n">
-        <v>363</v>
+        <v>3405</v>
       </c>
       <c r="I194" s="133" t="n">
-        <v>3570</v>
+        <v>640</v>
       </c>
       <c r="J194" s="134" t="n">
-        <v>2458.12</v>
+        <v>237.96</v>
       </c>
       <c r="K194" s="134" t="n">
-        <v>1814</v>
-      </c>
-      <c r="L194" s="236">
+        <v>238.12</v>
+      </c>
+      <c r="L194" s="237">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -18665,31 +18650,31 @@
       <c r="C195" s="135" t="n"/>
       <c r="D195" s="132" t="inlineStr">
         <is>
-          <t>台燿(6274)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G195" s="133" t="n">
-        <v>3635</v>
+        <v>3933</v>
       </c>
       <c r="H195" s="133" t="n">
-        <v>188</v>
+        <v>363</v>
       </c>
       <c r="I195" s="133" t="n">
-        <v>3447</v>
+        <v>3570</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>1398.04</v>
+        <v>2458.12</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>1878</v>
-      </c>
-      <c r="L195" s="237">
+        <v>1814</v>
+      </c>
+      <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -18700,29 +18685,29 @@
       <c r="C196" s="135" t="n"/>
       <c r="D196" s="132" t="inlineStr">
         <is>
-          <t>穩懋(3105)</t>
+          <t>台燿(6274)</t>
         </is>
       </c>
       <c r="E196" s="133" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="F196" s="133" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="G196" s="133" t="n">
-        <v>3365</v>
+        <v>3635</v>
       </c>
       <c r="H196" s="133" t="n">
-        <v>1713</v>
+        <v>188</v>
       </c>
       <c r="I196" s="133" t="n">
-        <v>1652</v>
+        <v>3447</v>
       </c>
       <c r="J196" s="134" t="n">
-        <v>467.4</v>
+        <v>1398.04</v>
       </c>
       <c r="K196" s="134" t="n">
-        <v>475.83</v>
+        <v>1878</v>
       </c>
       <c r="L196" s="237">
         <f>F196*(K196-J196)</f>
@@ -18735,29 +18720,29 @@
       <c r="C197" s="135" t="n"/>
       <c r="D197" s="132" t="inlineStr">
         <is>
-          <t>光寶科(2301)</t>
+          <t>穩懋(3105)</t>
         </is>
       </c>
       <c r="E197" s="133" t="n">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="F197" s="133" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G197" s="133" t="n">
-        <v>2832</v>
+        <v>3365</v>
       </c>
       <c r="H197" s="133" t="n">
-        <v>918</v>
+        <v>1713</v>
       </c>
       <c r="I197" s="133" t="n">
-        <v>1914</v>
+        <v>1652</v>
       </c>
       <c r="J197" s="134" t="n">
-        <v>314.68</v>
+        <v>467.4</v>
       </c>
       <c r="K197" s="134" t="n">
-        <v>316.52</v>
+        <v>475.83</v>
       </c>
       <c r="L197" s="237">
         <f>F197*(K197-J197)</f>
@@ -18770,31 +18755,31 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>欣興(3037)</t>
+          <t>光寶科(2301)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>2550</v>
+        <v>2832</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>1919</v>
+        <v>918</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>631</v>
+        <v>1914</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>980.65</v>
+        <v>314.68</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>959.6</v>
-      </c>
-      <c r="L198" s="236">
+        <v>316.52</v>
+      </c>
+      <c r="L198" s="237">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -29258,7 +29243,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 21:38 TW | 9/9 success | 來源: 富邦9/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-02 22:56 TW | 9/9 success | 來源: 富邦9/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-03 03:16
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="22">
+  <numFmts count="23">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -45,6 +45,7 @@
     <numFmt numFmtId="183" formatCode="&quot;📅 明日預測 ↕ 中性 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
     <numFmt numFmtId="184" formatCode="0&quot; 檔 +121億 &quot;&quot;(昨12/5d11)&quot;"/>
     <numFmt numFmtId="185" formatCode="0.0%&quot; 市-1608億 &quot;&quot;(昨21/5d19)&quot;"/>
+    <numFmt numFmtId="186" formatCode="0.0%&quot; 市-1614億 &quot;&quot;(昨21/5d19)&quot;"/>
   </numFmts>
   <fonts count="53">
     <font>
@@ -615,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="256">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1214,6 +1215,9 @@
     <xf numFmtId="185" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="186" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1899,10 +1903,10 @@
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
@@ -1929,10 +1933,10 @@
         <v>40732</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>268406</v>
+        <v>256864</v>
       </c>
     </row>
     <row r="18">
@@ -2667,23 +2671,23 @@
         <v>10</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
+          <t>強森</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="n">
+        <v>1370</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H32" s="17" t="n">
-        <v>2382</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>強森</t>
-        </is>
-      </c>
       <c r="J32" s="18" t="n">
-        <v>1370</v>
+        <v>949</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2697,7 +2701,7 @@
         <v>7</v>
       </c>
       <c r="N32" s="17" t="n">
-        <v>6618</v>
+        <v>5185</v>
       </c>
     </row>
     <row r="33">
@@ -2766,10 +2770,10 @@
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G34" s="16" t="inlineStr">
         <is>
@@ -2796,10 +2800,10 @@
         <v>132</v>
       </c>
       <c r="M34" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N34" s="17" t="n">
-        <v>1667</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2824,7 +2828,7 @@
         </is>
       </c>
       <c r="G37" s="244" t="n">
-        <v>-148.32073</v>
+        <v>-151.23464</v>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
@@ -2833,7 +2837,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C38" s="254" t="n">
+      <c r="C38" s="245" t="n">
         <v>19</v>
       </c>
       <c r="F38" s="22" t="inlineStr">
@@ -2841,8 +2845,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G38" s="255" t="n">
-        <v>0.2035157242394799</v>
+      <c r="G38" s="256" t="n">
+        <v>0.2029313523982471</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
@@ -2925,7 +2929,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2953,11 +2957,11 @@
         </is>
       </c>
       <c r="D45" s="33" t="n">
-        <v>951729</v>
+        <v>929828</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>20.6%</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2969,7 +2973,7 @@
         </is>
       </c>
       <c r="H45" s="33" t="n">
-        <v>268406</v>
+        <v>256864</v>
       </c>
       <c r="I45" s="234" t="n">
         <v>-0.009300000000000001</v>
@@ -2989,7 +2993,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -3021,7 +3025,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -3053,7 +3057,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.7%</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -3221,22 +3225,22 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 5 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>4 檔</t>
+          <t>5 檔</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3252,7 @@
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D58" s="40" t="inlineStr">
@@ -3258,7 +3262,7 @@
       </c>
       <c r="E58" s="40" t="inlineStr">
         <is>
-          <t>竹科主力分點 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F58" s="40" t="inlineStr">
@@ -3275,7 +3279,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>蔣承翰</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3285,7 +3289,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>蔣承翰 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>竹科主力分點 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3302,7 +3306,7 @@
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>蔣承翰</t>
         </is>
       </c>
       <c r="D60" s="40" t="inlineStr">
@@ -3312,7 +3316,7 @@
       </c>
       <c r="E60" s="40" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 4 檔新標的 (過去從沒買過)</t>
+          <t>蔣承翰 今日買進 4 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F60" s="40" t="inlineStr">
@@ -3656,7 +3660,7 @@
         </is>
       </c>
       <c r="C77" s="33" t="n">
-        <v>900821</v>
+        <v>877076</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3683,7 +3687,7 @@
         <v>76726</v>
       </c>
       <c r="J77" s="213" t="n">
-        <v>0.28286672585709</v>
+        <v>0.2905248472737998</v>
       </c>
     </row>
     <row r="78">
@@ -5401,7 +5405,7 @@
     <row r="9">
       <c r="C9" s="66" t="inlineStr">
         <is>
-          <t>② 聯發科 (2454) · 11 大戶</t>
+          <t>② 聯發科 (2454) · 10 大戶</t>
         </is>
       </c>
     </row>
@@ -5513,7 +5517,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-148 億 淨買</t>
+          <t>-151 億 淨買</t>
         </is>
       </c>
     </row>
@@ -18440,29 +18444,29 @@
       </c>
       <c r="D189" s="132" t="inlineStr">
         <is>
-          <t>聯發科(2454)</t>
+          <t>全新(2455)</t>
         </is>
       </c>
       <c r="E189" s="133" t="n">
-        <v>50</v>
+        <v>276</v>
       </c>
       <c r="F189" s="133" t="n">
-        <v>23</v>
+        <v>245</v>
       </c>
       <c r="G189" s="133" t="n">
-        <v>21375</v>
+        <v>14958</v>
       </c>
       <c r="H189" s="133" t="n">
-        <v>9832</v>
+        <v>13291</v>
       </c>
       <c r="I189" s="133" t="n">
-        <v>11543</v>
+        <v>1667</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>4275</v>
+        <v>541.97</v>
       </c>
       <c r="K189" s="134" t="n">
-        <v>4275</v>
+        <v>542.49</v>
       </c>
       <c r="L189" s="237">
         <f>F189*(K189-J189)</f>
@@ -18475,29 +18479,29 @@
       <c r="C190" s="135" t="n"/>
       <c r="D190" s="132" t="inlineStr">
         <is>
-          <t>全新(2455)</t>
+          <t>華星光(4979)</t>
         </is>
       </c>
       <c r="E190" s="133" t="n">
-        <v>276</v>
+        <v>90</v>
       </c>
       <c r="F190" s="133" t="n">
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="G190" s="133" t="n">
-        <v>14958</v>
+        <v>5539</v>
       </c>
       <c r="H190" s="133" t="n">
-        <v>13291</v>
+        <v>0</v>
       </c>
       <c r="I190" s="133" t="n">
-        <v>1667</v>
+        <v>5539</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>541.97</v>
+        <v>615.4</v>
       </c>
       <c r="K190" s="134" t="n">
-        <v>542.49</v>
+        <v>0</v>
       </c>
       <c r="L190" s="237">
         <f>F190*(K190-J190)</f>
@@ -18510,29 +18514,29 @@
       <c r="C191" s="135" t="n"/>
       <c r="D191" s="132" t="inlineStr">
         <is>
-          <t>華星光(4979)</t>
+          <t>禾伸堂(3026)</t>
         </is>
       </c>
       <c r="E191" s="133" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="F191" s="133" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G191" s="133" t="n">
-        <v>5539</v>
+        <v>4669</v>
       </c>
       <c r="H191" s="133" t="n">
-        <v>0</v>
+        <v>1652</v>
       </c>
       <c r="I191" s="133" t="n">
-        <v>5539</v>
+        <v>3017</v>
       </c>
       <c r="J191" s="134" t="n">
-        <v>622.3099999999999</v>
+        <v>686.62</v>
       </c>
       <c r="K191" s="134" t="n">
-        <v>0</v>
+        <v>688.33</v>
       </c>
       <c r="L191" s="237">
         <f>F191*(K191-J191)</f>
@@ -18545,29 +18549,29 @@
       <c r="C192" s="135" t="n"/>
       <c r="D192" s="132" t="inlineStr">
         <is>
-          <t>禾伸堂(3026)</t>
+          <t>台光電(2383)</t>
         </is>
       </c>
       <c r="E192" s="133" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="F192" s="133" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G192" s="133" t="n">
-        <v>4669</v>
+        <v>4447</v>
       </c>
       <c r="H192" s="133" t="n">
-        <v>1652</v>
+        <v>0</v>
       </c>
       <c r="I192" s="133" t="n">
-        <v>3017</v>
+        <v>4447</v>
       </c>
       <c r="J192" s="134" t="n">
-        <v>686.62</v>
+        <v>5559.12</v>
       </c>
       <c r="K192" s="134" t="n">
-        <v>688.33</v>
+        <v>0</v>
       </c>
       <c r="L192" s="237">
         <f>F192*(K192-J192)</f>
@@ -18580,29 +18584,29 @@
       <c r="C193" s="135" t="n"/>
       <c r="D193" s="132" t="inlineStr">
         <is>
-          <t>台光電(2383)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E193" s="133" t="n">
-        <v>8</v>
+        <v>170</v>
       </c>
       <c r="F193" s="133" t="n">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="G193" s="133" t="n">
-        <v>4447</v>
+        <v>4045</v>
       </c>
       <c r="H193" s="133" t="n">
-        <v>0</v>
+        <v>3405</v>
       </c>
       <c r="I193" s="133" t="n">
-        <v>4447</v>
+        <v>640</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>5559.12</v>
+        <v>237.96</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>0</v>
+        <v>238.12</v>
       </c>
       <c r="L193" s="237">
         <f>F193*(K193-J193)</f>
@@ -18615,31 +18619,31 @@
       <c r="C194" s="135" t="n"/>
       <c r="D194" s="132" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E194" s="133" t="n">
-        <v>170</v>
+        <v>16</v>
       </c>
       <c r="F194" s="133" t="n">
-        <v>143</v>
+        <v>2</v>
       </c>
       <c r="G194" s="133" t="n">
-        <v>4045</v>
+        <v>3933</v>
       </c>
       <c r="H194" s="133" t="n">
-        <v>3405</v>
+        <v>363</v>
       </c>
       <c r="I194" s="133" t="n">
-        <v>640</v>
+        <v>3570</v>
       </c>
       <c r="J194" s="134" t="n">
-        <v>237.96</v>
+        <v>2458.12</v>
       </c>
       <c r="K194" s="134" t="n">
-        <v>238.12</v>
-      </c>
-      <c r="L194" s="237">
+        <v>1814</v>
+      </c>
+      <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -18650,31 +18654,31 @@
       <c r="C195" s="135" t="n"/>
       <c r="D195" s="132" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>台燿(6274)</t>
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G195" s="133" t="n">
-        <v>3933</v>
+        <v>3635</v>
       </c>
       <c r="H195" s="133" t="n">
-        <v>363</v>
+        <v>188</v>
       </c>
       <c r="I195" s="133" t="n">
-        <v>3570</v>
+        <v>3447</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>2458.12</v>
+        <v>1398.04</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>1814</v>
-      </c>
-      <c r="L195" s="236">
+        <v>1878</v>
+      </c>
+      <c r="L195" s="237">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -18685,29 +18689,29 @@
       <c r="C196" s="135" t="n"/>
       <c r="D196" s="132" t="inlineStr">
         <is>
-          <t>台燿(6274)</t>
+          <t>穩懋(3105)</t>
         </is>
       </c>
       <c r="E196" s="133" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="F196" s="133" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="G196" s="133" t="n">
-        <v>3635</v>
+        <v>3365</v>
       </c>
       <c r="H196" s="133" t="n">
-        <v>188</v>
+        <v>1713</v>
       </c>
       <c r="I196" s="133" t="n">
-        <v>3447</v>
+        <v>1652</v>
       </c>
       <c r="J196" s="134" t="n">
-        <v>1398.04</v>
+        <v>467.4</v>
       </c>
       <c r="K196" s="134" t="n">
-        <v>1878</v>
+        <v>475.83</v>
       </c>
       <c r="L196" s="237">
         <f>F196*(K196-J196)</f>
@@ -18720,29 +18724,29 @@
       <c r="C197" s="135" t="n"/>
       <c r="D197" s="132" t="inlineStr">
         <is>
-          <t>穩懋(3105)</t>
+          <t>光寶科(2301)</t>
         </is>
       </c>
       <c r="E197" s="133" t="n">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="F197" s="133" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="G197" s="133" t="n">
-        <v>3365</v>
+        <v>2832</v>
       </c>
       <c r="H197" s="133" t="n">
-        <v>1713</v>
+        <v>918</v>
       </c>
       <c r="I197" s="133" t="n">
-        <v>1652</v>
+        <v>1914</v>
       </c>
       <c r="J197" s="134" t="n">
-        <v>467.4</v>
+        <v>314.68</v>
       </c>
       <c r="K197" s="134" t="n">
-        <v>475.83</v>
+        <v>316.52</v>
       </c>
       <c r="L197" s="237">
         <f>F197*(K197-J197)</f>
@@ -18755,31 +18759,31 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>光寶科(2301)</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>2832</v>
+        <v>2550</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>918</v>
+        <v>1919</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>1914</v>
+        <v>631</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>314.68</v>
+        <v>980.65</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>316.52</v>
-      </c>
-      <c r="L198" s="237">
+        <v>959.6</v>
+      </c>
+      <c r="L198" s="236">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -29243,7 +29247,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-03 02:19 TW | 9/9 success | 來源: 富邦9/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-03 03:16 TW | 9/9 success | 來源: 富邦9/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-03 22:54
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -2027,7 +2027,7 @@
         <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>38483</v>
+        <v>39193</v>
       </c>
     </row>
     <row r="21">
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="G32" s="257" t="n">
-        <v>-199.32547</v>
+        <v>-199.54917</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
@@ -2559,7 +2559,7 @@
         </is>
       </c>
       <c r="G33" s="259" t="n">
-        <v>0.1702456257638463</v>
+        <v>0.1707376082472423</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2670,11 +2670,11 @@
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>870535</v>
+        <v>881453</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -3213,7 +3213,7 @@
         </is>
       </c>
       <c r="C66" s="33" t="n">
-        <v>809114</v>
+        <v>819686</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3240,7 +3240,7 @@
         <v>40121</v>
       </c>
       <c r="J66" s="213" t="n">
-        <v>0.2024861026965552</v>
+        <v>0.199874464124067</v>
       </c>
     </row>
     <row r="67">
@@ -5098,7 +5098,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-199 億 淨買</t>
+          <t>-200 億 淨買</t>
         </is>
       </c>
     </row>
@@ -17570,7 +17570,7 @@
         </is>
       </c>
       <c r="E189" s="133" t="n">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F189" s="133" t="n">
         <v>4</v>
@@ -17585,7 +17585,7 @@
         <v>36163</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>1344.34</v>
+        <v>1349.28</v>
       </c>
       <c r="K189" s="134" t="n">
         <v>1342.5</v>
@@ -17605,10 +17605,10 @@
         </is>
       </c>
       <c r="E190" s="133" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F190" s="133" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G190" s="133" t="n">
         <v>6900</v>
@@ -17620,10 +17620,10 @@
         <v>5108</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>425.9</v>
+        <v>413.15</v>
       </c>
       <c r="K190" s="134" t="n">
-        <v>448.05</v>
+        <v>416.79</v>
       </c>
       <c r="L190" s="237">
         <f>F190*(K190-J190)</f>
@@ -17640,7 +17640,7 @@
         </is>
       </c>
       <c r="E191" s="133" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F191" s="133" t="n">
         <v>15</v>
@@ -17655,7 +17655,7 @@
         <v>5017</v>
       </c>
       <c r="J191" s="134" t="n">
-        <v>478.7</v>
+        <v>470.85</v>
       </c>
       <c r="K191" s="134" t="n">
         <v>484.53</v>
@@ -17710,10 +17710,10 @@
         </is>
       </c>
       <c r="E193" s="133" t="n">
-        <v>101</v>
+        <v>195</v>
       </c>
       <c r="F193" s="133" t="n">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="G193" s="133" t="n">
         <v>4975</v>
@@ -17725,12 +17725,12 @@
         <v>2627</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>492.6</v>
+        <v>255.14</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>521.67</v>
-      </c>
-      <c r="L193" s="237">
+        <v>194.01</v>
+      </c>
+      <c r="L193" s="236">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -17745,10 +17745,10 @@
         </is>
       </c>
       <c r="E194" s="133" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F194" s="133" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G194" s="133" t="n">
         <v>4190</v>
@@ -17760,12 +17760,12 @@
         <v>3002</v>
       </c>
       <c r="J194" s="134" t="n">
-        <v>654.66</v>
+        <v>634.8200000000001</v>
       </c>
       <c r="K194" s="134" t="n">
-        <v>698.53</v>
-      </c>
-      <c r="L194" s="237">
+        <v>625</v>
+      </c>
+      <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -17780,10 +17780,10 @@
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G195" s="133" t="n">
         <v>3951</v>
@@ -17795,10 +17795,10 @@
         <v>2153</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>1067.78</v>
+        <v>940.67</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>1057.65</v>
+        <v>899</v>
       </c>
       <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
@@ -17881,29 +17881,29 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>富喬(1815)</t>
+          <t>晶豪科(3006)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>237</v>
+        <v>111</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>2864</v>
+        <v>3075</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>441</v>
+        <v>2493</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>2423</v>
+        <v>582</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>120.84</v>
+        <v>277</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>126</v>
+        <v>277</v>
       </c>
       <c r="L198" s="237">
         <f>F198*(K198-J198)</f>
@@ -28138,7 +28138,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-03 21:37 TW | 1/1 success | 來源: 富邦1/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-03 22:54 TW | 1/1 success | 來源: 富邦1/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-04 01:22
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -52,7 +52,7 @@
     <numFmt numFmtId="189" formatCode="0.0%&quot; 市-1215億 &quot;&quot;(昨20/5d18)&quot;"/>
     <numFmt numFmtId="190" formatCode="&quot;📅 明日預測 ↓ 偏空 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 1 檔焦點&quot;"/>
   </numFmts>
-  <fonts count="54">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -362,6 +362,12 @@
       <color rgb="FF059669"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Noto Sans TC"/>
+      <i val="1"/>
+      <color rgb="FF10B981"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="51">
     <fill>
@@ -633,7 +639,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="262">
+  <cellXfs count="263">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1248,6 +1254,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="53" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1635,7 +1642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N131"/>
+  <dimension ref="B2:N118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1671,7 +1678,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2408 / 6669 / 8046 (Q5 偏空, 中性信號)  |  避開 — 除權息 4 檔: 1203, 3661, 7780 ... | 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏空 (Q5 10%, hot=14)</t>
+          <t>💡 📌 一般共識 2408 / 6669 / 8046 (Q5 偏空, 中性信號)  |  避開 — 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏空 (Q5 10%, hot=14)</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2566,7 @@
         </is>
       </c>
       <c r="G33" s="259" t="n">
-        <v>0.1707376082472423</v>
+        <v>0.1706536496408914</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -3690,7 +3697,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="B80" s="57" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260902)</t>
+          <t>▍ G. 注意股 (資料日 20260904)</t>
         </is>
       </c>
     </row>
@@ -3722,1108 +3729,794 @@
       </c>
     </row>
     <row r="82">
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>066185</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>聯發科元大64購05</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
-        <v>1</v>
-      </c>
-      <c r="E82" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="40" t="inlineStr">
-        <is>
-          <t>069544</t>
-        </is>
-      </c>
-      <c r="C83" s="40" t="inlineStr">
-        <is>
-          <t>立隆電元大5B購05</t>
-        </is>
-      </c>
-      <c r="D83" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" s="40" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="F83" s="40" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>2426</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>鼎元</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>1</v>
-      </c>
-      <c r="E84" t="n">
-        <v>104.5</v>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>1045.00</t>
+      <c r="B82" s="262" t="inlineStr">
+        <is>
+          <t>✅ 今日無新增注意股 (市場無異常波動標的)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>▍ H. 借券賣出 Top 15 (機構級反向力量, 資料日 20260903)</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="B85" s="40" t="inlineStr">
-        <is>
-          <t>2455</t>
-        </is>
-      </c>
-      <c r="C85" s="40" t="inlineStr">
-        <is>
-          <t>全新</t>
-        </is>
-      </c>
-      <c r="D85" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E85" s="40" t="n">
-        <v>542</v>
-      </c>
-      <c r="F85" s="40" t="inlineStr">
-        <is>
-          <t>132.84</t>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>名稱</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>借券張數</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>融券張數</t>
+        </is>
+      </c>
+      <c r="F85" s="12" t="inlineStr">
+        <is>
+          <t>ratio</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>2466</t>
+          <t>2887</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>冠西電</t>
-        </is>
-      </c>
-      <c r="D86" t="n">
-        <v>1</v>
-      </c>
-      <c r="E86" t="n">
-        <v>104</v>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>66.24</t>
-        </is>
+          <t>台新新光金</t>
+        </is>
+      </c>
+      <c r="D86" s="33" t="n">
+        <v>15554</v>
+      </c>
+      <c r="E86" s="33" t="n">
+        <v>107</v>
+      </c>
+      <c r="F86" s="215" t="n">
+        <v>145.36</v>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="40" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>2344</t>
         </is>
       </c>
       <c r="C87" s="40" t="inlineStr">
         <is>
-          <t>大立光</t>
-        </is>
-      </c>
-      <c r="D87" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" s="40" t="n">
-        <v>7810</v>
-      </c>
-      <c r="F87" s="40" t="inlineStr">
-        <is>
-          <t>41.54</t>
-        </is>
+          <t>華邦電</t>
+        </is>
+      </c>
+      <c r="D87" s="60" t="n">
+        <v>10700</v>
+      </c>
+      <c r="E87" s="60" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F87" s="216" t="n">
+        <v>2.23</v>
       </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>3406</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>玉晶光</t>
-        </is>
-      </c>
-      <c r="D88" t="n">
-        <v>1</v>
-      </c>
-      <c r="E88" t="n">
-        <v>1050</v>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>28.41</t>
-        </is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="D88" s="33" t="n">
+        <v>7573</v>
+      </c>
+      <c r="E88" s="33" t="n">
+        <v>1609</v>
+      </c>
+      <c r="F88" s="215" t="n">
+        <v>4.71</v>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="40" t="inlineStr">
         <is>
-          <t>3450</t>
+          <t>2883</t>
         </is>
       </c>
       <c r="C89" s="40" t="inlineStr">
         <is>
-          <t>聯鈞</t>
-        </is>
-      </c>
-      <c r="D89" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E89" s="40" t="n">
-        <v>602</v>
-      </c>
-      <c r="F89" s="40" t="inlineStr">
-        <is>
-          <t>122.11</t>
-        </is>
+          <t>凱基金</t>
+        </is>
+      </c>
+      <c r="D89" s="60" t="n">
+        <v>6933</v>
+      </c>
+      <c r="E89" s="60" t="n">
+        <v>52</v>
+      </c>
+      <c r="F89" s="216" t="n">
+        <v>133.33</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>6226</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>光鼎</t>
-        </is>
-      </c>
-      <c r="D90" t="n">
-        <v>1</v>
-      </c>
-      <c r="E90" t="n">
-        <v>34.15</v>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
+          <t>力積電</t>
+        </is>
+      </c>
+      <c r="D90" s="33" t="n">
+        <v>6755</v>
+      </c>
+      <c r="E90" s="33" t="n">
+        <v>269</v>
+      </c>
+      <c r="F90" s="215" t="n">
+        <v>25.11</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="40" t="inlineStr">
         <is>
-          <t>6834</t>
+          <t>2449</t>
         </is>
       </c>
       <c r="C91" s="40" t="inlineStr">
         <is>
-          <t>天二科技</t>
-        </is>
-      </c>
-      <c r="D91" s="40" t="n">
+          <t>京元電子</t>
+        </is>
+      </c>
+      <c r="D91" s="60" t="n">
+        <v>5779</v>
+      </c>
+      <c r="E91" s="60" t="n">
+        <v>26</v>
+      </c>
+      <c r="F91" s="216" t="n">
+        <v>222.27</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="43" t="inlineStr">
+        <is>
+          <t>🔴 00918</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>大華優利高填息30</t>
+        </is>
+      </c>
+      <c r="D92" s="33" t="n">
+        <v>4933</v>
+      </c>
+      <c r="E92" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="E91" s="40" t="n">
-        <v>92.2</v>
-      </c>
-      <c r="F91" s="40" t="inlineStr">
-        <is>
-          <t>40.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>6933</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>AMAX-KY</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
-        <v>1</v>
-      </c>
-      <c r="E92" t="n">
-        <v>331</v>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>41.07</t>
-        </is>
+      <c r="F92" s="252" t="n">
+        <v>4933</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="40" t="inlineStr">
         <is>
-          <t>8039</t>
+          <t>2891</t>
         </is>
       </c>
       <c r="C93" s="40" t="inlineStr">
         <is>
-          <t>台虹</t>
-        </is>
-      </c>
-      <c r="D93" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E93" s="40" t="n">
-        <v>313.5</v>
-      </c>
-      <c r="F93" s="40" t="inlineStr">
-        <is>
-          <t>99.52</t>
-        </is>
+          <t>中信金</t>
+        </is>
+      </c>
+      <c r="D93" s="60" t="n">
+        <v>4673</v>
+      </c>
+      <c r="E93" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="F93" s="216" t="n">
+        <v>259.61</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>8473</t>
+          <t>00685L</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>山林水</t>
-        </is>
-      </c>
-      <c r="D94" t="n">
-        <v>1</v>
-      </c>
-      <c r="E94" t="n">
-        <v>45.95</v>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>13.32</t>
-        </is>
+          <t>群益臺灣加權正2</t>
+        </is>
+      </c>
+      <c r="D94" s="33" t="n">
+        <v>3808</v>
+      </c>
+      <c r="E94" s="33" t="n">
+        <v>1685</v>
+      </c>
+      <c r="F94" s="215" t="n">
+        <v>2.26</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="40" t="inlineStr">
         <is>
-          <t>911608</t>
+          <t>1802</t>
         </is>
       </c>
       <c r="C95" s="40" t="inlineStr">
         <is>
-          <t>明輝-DR</t>
-        </is>
-      </c>
-      <c r="D95" s="40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E95" s="40" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="F95" s="40" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="22" customHeight="1">
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>▍ H. 借券賣出 Top 15 (機構級反向力量, 資料日 20260903)</t>
-        </is>
+          <t>台玻</t>
+        </is>
+      </c>
+      <c r="D95" s="60" t="n">
+        <v>3247</v>
+      </c>
+      <c r="E95" s="60" t="n">
+        <v>493</v>
+      </c>
+      <c r="F95" s="216" t="n">
+        <v>6.59</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1303</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>南亞</t>
+        </is>
+      </c>
+      <c r="D96" s="33" t="n">
+        <v>3236</v>
+      </c>
+      <c r="E96" s="33" t="n">
+        <v>131</v>
+      </c>
+      <c r="F96" s="215" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="40" t="inlineStr">
+        <is>
+          <t>3231</t>
+        </is>
+      </c>
+      <c r="C97" s="40" t="inlineStr">
+        <is>
+          <t>緯創</t>
+        </is>
+      </c>
+      <c r="D97" s="60" t="n">
+        <v>3177</v>
+      </c>
+      <c r="E97" s="60" t="n">
+        <v>113</v>
+      </c>
+      <c r="F97" s="216" t="n">
+        <v>28.12</v>
       </c>
     </row>
     <row r="98">
-      <c r="B98" s="12" t="inlineStr">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>00981A</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>主動統一台股增長</t>
+        </is>
+      </c>
+      <c r="D98" s="33" t="n">
+        <v>2866</v>
+      </c>
+      <c r="E98" s="33" t="n">
+        <v>184</v>
+      </c>
+      <c r="F98" s="215" t="n">
+        <v>15.58</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="44" t="inlineStr">
+        <is>
+          <t>🔴 1718</t>
+        </is>
+      </c>
+      <c r="C99" s="40" t="inlineStr">
+        <is>
+          <t>中纖</t>
+        </is>
+      </c>
+      <c r="D99" s="60" t="n">
+        <v>2794</v>
+      </c>
+      <c r="E99" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" s="217" t="n">
+        <v>1397</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2426</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>鼎元</t>
+        </is>
+      </c>
+      <c r="D100" s="33" t="n">
+        <v>2695</v>
+      </c>
+      <c r="E100" s="33" t="n">
+        <v>456</v>
+      </c>
+      <c r="F100" s="215" t="n">
+        <v>5.91</v>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="B102" s="62" t="inlineStr">
+        <is>
+          <t>▍ I. 未來 30 天除權息 (有效 74 檔, 已剔除過期)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="58" t="inlineStr">
+        <is>
+          <t>除權息日</t>
+        </is>
+      </c>
+      <c r="C103" s="58" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C98" s="12" t="inlineStr">
+      <c r="D103" s="58" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D98" s="12" t="inlineStr">
-        <is>
-          <t>借券張數</t>
-        </is>
-      </c>
-      <c r="E98" s="12" t="inlineStr">
-        <is>
-          <t>融券張數</t>
-        </is>
-      </c>
-      <c r="F98" s="12" t="inlineStr">
-        <is>
-          <t>ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>2887</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>台新新光金</t>
-        </is>
-      </c>
-      <c r="D99" s="33" t="n">
-        <v>15554</v>
-      </c>
-      <c r="E99" s="33" t="n">
-        <v>107</v>
-      </c>
-      <c r="F99" s="215" t="n">
-        <v>145.36</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="B100" s="40" t="inlineStr">
-        <is>
-          <t>2344</t>
-        </is>
-      </c>
-      <c r="C100" s="40" t="inlineStr">
-        <is>
-          <t>華邦電</t>
-        </is>
-      </c>
-      <c r="D100" s="60" t="n">
-        <v>10700</v>
-      </c>
-      <c r="E100" s="60" t="n">
-        <v>4800</v>
-      </c>
-      <c r="F100" s="216" t="n">
-        <v>2.23</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>2408</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>南亞科</t>
-        </is>
-      </c>
-      <c r="D101" s="33" t="n">
-        <v>7573</v>
-      </c>
-      <c r="E101" s="33" t="n">
-        <v>1609</v>
-      </c>
-      <c r="F101" s="215" t="n">
-        <v>4.71</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="B102" s="40" t="inlineStr">
-        <is>
-          <t>2883</t>
-        </is>
-      </c>
-      <c r="C102" s="40" t="inlineStr">
-        <is>
-          <t>凱基金</t>
-        </is>
-      </c>
-      <c r="D102" s="60" t="n">
-        <v>6933</v>
-      </c>
-      <c r="E102" s="60" t="n">
-        <v>52</v>
-      </c>
-      <c r="F102" s="216" t="n">
-        <v>133.33</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>6770</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>力積電</t>
-        </is>
-      </c>
-      <c r="D103" s="33" t="n">
-        <v>6755</v>
-      </c>
-      <c r="E103" s="33" t="n">
-        <v>269</v>
-      </c>
-      <c r="F103" s="215" t="n">
-        <v>25.11</v>
+      <c r="E103" s="58" t="inlineStr">
+        <is>
+          <t>類型</t>
+        </is>
+      </c>
+      <c r="F103" s="58" t="inlineStr">
+        <is>
+          <t>現金股利</t>
+        </is>
       </c>
     </row>
     <row r="104">
-      <c r="B104" s="40" t="inlineStr">
-        <is>
-          <t>2449</t>
-        </is>
-      </c>
-      <c r="C104" s="40" t="inlineStr">
-        <is>
-          <t>京元電子</t>
-        </is>
-      </c>
-      <c r="D104" s="60" t="n">
-        <v>5779</v>
-      </c>
-      <c r="E104" s="60" t="n">
-        <v>26</v>
-      </c>
-      <c r="F104" s="216" t="n">
-        <v>222.27</v>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>20260907</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>00400A</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>主動國泰動能高息</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>0.12</v>
       </c>
     </row>
     <row r="105">
-      <c r="B105" s="43" t="inlineStr">
-        <is>
-          <t>🔴 00918</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>大華優利高填息30</t>
-        </is>
-      </c>
-      <c r="D105" s="33" t="n">
-        <v>4933</v>
-      </c>
-      <c r="E105" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="F105" s="252" t="n">
-        <v>4933</v>
+      <c r="B105" s="40" t="inlineStr">
+        <is>
+          <t>20260907</t>
+        </is>
+      </c>
+      <c r="C105" s="40" t="inlineStr">
+        <is>
+          <t>01010T</t>
+        </is>
+      </c>
+      <c r="D105" s="40" t="inlineStr">
+        <is>
+          <t>京城樂富R1</t>
+        </is>
+      </c>
+      <c r="E105" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F105" s="40" t="n">
+        <v>0.09872</v>
       </c>
     </row>
     <row r="106">
-      <c r="B106" s="40" t="inlineStr">
-        <is>
-          <t>2891</t>
-        </is>
-      </c>
-      <c r="C106" s="40" t="inlineStr">
-        <is>
-          <t>中信金</t>
-        </is>
-      </c>
-      <c r="D106" s="60" t="n">
-        <v>4673</v>
-      </c>
-      <c r="E106" s="60" t="n">
-        <v>18</v>
-      </c>
-      <c r="F106" s="216" t="n">
-        <v>259.61</v>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>20260907</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>1466</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>聚隆</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="107">
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>00685L</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>群益臺灣加權正2</t>
-        </is>
-      </c>
-      <c r="D107" s="33" t="n">
-        <v>3808</v>
-      </c>
-      <c r="E107" s="33" t="n">
-        <v>1685</v>
-      </c>
-      <c r="F107" s="215" t="n">
-        <v>2.26</v>
+      <c r="B107" s="40" t="inlineStr">
+        <is>
+          <t>20260907</t>
+        </is>
+      </c>
+      <c r="C107" s="40" t="inlineStr">
+        <is>
+          <t>6533</t>
+        </is>
+      </c>
+      <c r="D107" s="40" t="inlineStr">
+        <is>
+          <t>晶心科</t>
+        </is>
+      </c>
+      <c r="E107" s="40" t="inlineStr">
+        <is>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F107" s="40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="108">
-      <c r="B108" s="40" t="inlineStr">
-        <is>
-          <t>1802</t>
-        </is>
-      </c>
-      <c r="C108" s="40" t="inlineStr">
-        <is>
-          <t>台玻</t>
-        </is>
-      </c>
-      <c r="D108" s="60" t="n">
-        <v>3247</v>
-      </c>
-      <c r="E108" s="60" t="n">
-        <v>493</v>
-      </c>
-      <c r="F108" s="216" t="n">
-        <v>6.59</v>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>00940</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>元大台灣價值高息</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
       </c>
     </row>
     <row r="109">
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>1303</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>南亞</t>
-        </is>
-      </c>
-      <c r="D109" s="33" t="n">
-        <v>3236</v>
-      </c>
-      <c r="E109" s="33" t="n">
-        <v>131</v>
-      </c>
-      <c r="F109" s="215" t="n">
-        <v>24.7</v>
+      <c r="B109" s="40" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C109" s="40" t="inlineStr">
+        <is>
+          <t>2379</t>
+        </is>
+      </c>
+      <c r="D109" s="40" t="inlineStr">
+        <is>
+          <t>瑞昱</t>
+        </is>
+      </c>
+      <c r="E109" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F109" s="40" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="110">
-      <c r="B110" s="40" t="inlineStr">
-        <is>
-          <t>3231</t>
-        </is>
-      </c>
-      <c r="C110" s="40" t="inlineStr">
-        <is>
-          <t>緯創</t>
-        </is>
-      </c>
-      <c r="D110" s="60" t="n">
-        <v>3177</v>
-      </c>
-      <c r="E110" s="60" t="n">
-        <v>113</v>
-      </c>
-      <c r="F110" s="216" t="n">
-        <v>28.12</v>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2442</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>新美齊</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>2.031861</v>
       </c>
     </row>
     <row r="111">
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>00981A</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>主動統一台股增長</t>
-        </is>
-      </c>
-      <c r="D111" s="33" t="n">
-        <v>2866</v>
-      </c>
-      <c r="E111" s="33" t="n">
-        <v>184</v>
-      </c>
-      <c r="F111" s="215" t="n">
-        <v>15.58</v>
+      <c r="B111" s="40" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C111" s="40" t="inlineStr">
+        <is>
+          <t>2706</t>
+        </is>
+      </c>
+      <c r="D111" s="40" t="inlineStr">
+        <is>
+          <t>第一店</t>
+        </is>
+      </c>
+      <c r="E111" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F111" s="40" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="112">
-      <c r="B112" s="44" t="inlineStr">
-        <is>
-          <t>🔴 1718</t>
-        </is>
-      </c>
-      <c r="C112" s="40" t="inlineStr">
-        <is>
-          <t>中纖</t>
-        </is>
-      </c>
-      <c r="D112" s="60" t="n">
-        <v>2794</v>
-      </c>
-      <c r="E112" s="60" t="n">
-        <v>2</v>
-      </c>
-      <c r="F112" s="217" t="n">
-        <v>1397</v>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>3312</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>弘憶股</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="113">
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>2426</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>鼎元</t>
-        </is>
-      </c>
-      <c r="D113" s="33" t="n">
-        <v>2695</v>
-      </c>
-      <c r="E113" s="33" t="n">
-        <v>456</v>
-      </c>
-      <c r="F113" s="215" t="n">
-        <v>5.91</v>
-      </c>
-    </row>
-    <row r="115" ht="22" customHeight="1">
-      <c r="B115" s="62" t="inlineStr">
-        <is>
-          <t>▍ I. 未來 30 天除權息 (有效 77 檔, 已剔除過期)</t>
-        </is>
+      <c r="B113" s="40" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C113" s="40" t="inlineStr">
+        <is>
+          <t>3622</t>
+        </is>
+      </c>
+      <c r="D113" s="40" t="inlineStr">
+        <is>
+          <t>洋華</t>
+        </is>
+      </c>
+      <c r="E113" s="40" t="inlineStr">
+        <is>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F113" s="40" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>8473</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>山林水</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>0.782345</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="40" t="inlineStr">
+        <is>
+          <t>20260908</t>
+        </is>
+      </c>
+      <c r="C115" s="40" t="inlineStr">
+        <is>
+          <t>9933</t>
+        </is>
+      </c>
+      <c r="D115" s="40" t="inlineStr">
+        <is>
+          <t>中鼎</t>
+        </is>
+      </c>
+      <c r="E115" s="40" t="inlineStr">
+        <is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F115" s="40" t="n">
+        <v>0.763056</v>
       </c>
     </row>
     <row r="116">
-      <c r="B116" s="58" t="inlineStr">
-        <is>
-          <t>除權息日</t>
-        </is>
-      </c>
-      <c r="C116" s="58" t="inlineStr">
-        <is>
-          <t>代號</t>
-        </is>
-      </c>
-      <c r="D116" s="58" t="inlineStr">
-        <is>
-          <t>名稱</t>
-        </is>
-      </c>
-      <c r="E116" s="58" t="inlineStr">
-        <is>
-          <t>類型</t>
-        </is>
-      </c>
-      <c r="F116" s="58" t="inlineStr">
-        <is>
-          <t>現金股利</t>
-        </is>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>20260909</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>三地開發</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>權息</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="117">
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>20260903</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>1203</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>味王</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
+      <c r="B117" s="40" t="inlineStr">
+        <is>
+          <t>20260909</t>
+        </is>
+      </c>
+      <c r="C117" s="40" t="inlineStr">
+        <is>
+          <t>3059</t>
+        </is>
+      </c>
+      <c r="D117" s="40" t="inlineStr">
+        <is>
+          <t>華晶科</t>
+        </is>
+      </c>
+      <c r="E117" s="40" t="inlineStr">
         <is>
           <t>息</t>
         </is>
       </c>
-      <c r="F117" t="n">
-        <v>1</v>
+      <c r="F117" s="40" t="n">
+        <v>0.998614</v>
       </c>
     </row>
     <row r="118">
-      <c r="B118" s="40" t="inlineStr">
-        <is>
-          <t>20260903</t>
-        </is>
-      </c>
-      <c r="C118" s="40" t="inlineStr">
-        <is>
-          <t>3661</t>
-        </is>
-      </c>
-      <c r="D118" s="40" t="inlineStr">
-        <is>
-          <t>世芯-KY</t>
-        </is>
-      </c>
-      <c r="E118" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F118" s="40" t="n">
-        <v>32.551656</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>20260903</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>7780</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>大研生醫*</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F119" t="n">
-        <v>0.116588</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="40" t="inlineStr">
-        <is>
-          <t>20260903</t>
-        </is>
-      </c>
-      <c r="C120" s="40" t="inlineStr">
-        <is>
-          <t>8466</t>
-        </is>
-      </c>
-      <c r="D120" s="40" t="inlineStr">
-        <is>
-          <t>美吉吉-KY</t>
-        </is>
-      </c>
-      <c r="E120" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F120" s="40" t="n">
-        <v>0.301938</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>20260907</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>00400A</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>主動國泰動能高息</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F121" t="n">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="B122" s="40" t="inlineStr">
-        <is>
-          <t>20260907</t>
-        </is>
-      </c>
-      <c r="C122" s="40" t="inlineStr">
-        <is>
-          <t>01010T</t>
-        </is>
-      </c>
-      <c r="D122" s="40" t="inlineStr">
-        <is>
-          <t>京城樂富R1</t>
-        </is>
-      </c>
-      <c r="E122" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F122" s="40" t="n">
-        <v>0.09872</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>20260907</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>1466</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>聚隆</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F123" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="B124" s="40" t="inlineStr">
-        <is>
-          <t>20260907</t>
-        </is>
-      </c>
-      <c r="C124" s="40" t="inlineStr">
-        <is>
-          <t>6533</t>
-        </is>
-      </c>
-      <c r="D124" s="40" t="inlineStr">
-        <is>
-          <t>晶心科</t>
-        </is>
-      </c>
-      <c r="E124" s="40" t="inlineStr">
-        <is>
-          <t>權</t>
-        </is>
-      </c>
-      <c r="F124" s="40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>00940</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>元大台灣價值高息</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="B126" s="40" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C126" s="40" t="inlineStr">
-        <is>
-          <t>2379</t>
-        </is>
-      </c>
-      <c r="D126" s="40" t="inlineStr">
-        <is>
-          <t>瑞昱</t>
-        </is>
-      </c>
-      <c r="E126" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F126" s="40" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>2442</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>新美齊</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>20260909</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>3706</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>神達</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
         <is>
           <t>權息</t>
         </is>
       </c>
-      <c r="F127" t="n">
-        <v>2.031861</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="B128" s="40" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C128" s="40" t="inlineStr">
-        <is>
-          <t>2706</t>
-        </is>
-      </c>
-      <c r="D128" s="40" t="inlineStr">
-        <is>
-          <t>第一店</t>
-        </is>
-      </c>
-      <c r="E128" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F128" s="40" t="n">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>3312</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>弘憶股</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F129" t="n">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="B130" s="40" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C130" s="40" t="inlineStr">
-        <is>
-          <t>3622</t>
-        </is>
-      </c>
-      <c r="D130" s="40" t="inlineStr">
-        <is>
-          <t>洋華</t>
-        </is>
-      </c>
-      <c r="E130" s="40" t="inlineStr">
-        <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F130" s="40" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>20260908</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>8473</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>山林水</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>權息</t>
-        </is>
-      </c>
-      <c r="F131" t="n">
-        <v>0.782345</v>
+      <c r="F118" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="B9:N9"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="F37:I37"/>
     <mergeCell ref="G33:I33"/>
     <mergeCell ref="B35:N35"/>
     <mergeCell ref="B4:N4"/>
+    <mergeCell ref="B84:J84"/>
     <mergeCell ref="B7:N7"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="B64:J64"/>
+    <mergeCell ref="B82:F82"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="B80:J80"/>
     <mergeCell ref="B12:N12"/>
     <mergeCell ref="B11:N11"/>
-    <mergeCell ref="B97:J97"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B54:J54"/>
     <mergeCell ref="B14:N14"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="B8:N8"/>
     <mergeCell ref="B46:J46"/>
-    <mergeCell ref="B115:J115"/>
     <mergeCell ref="B13:N13"/>
     <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B102:J102"/>
     <mergeCell ref="B37:E37"/>
     <mergeCell ref="B34:N34"/>
     <mergeCell ref="B10:N10"/>
@@ -4900,17 +4593,8 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D82:D95">
+  <conditionalFormatting sqref="D86:D100">
     <cfRule type="dataBar" priority="9">
-      <dataBar minLength="5" maxLength="90" showValue="1">
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFB300"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D99:D113">
-    <cfRule type="dataBar" priority="10">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4918,8 +4602,8 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F99:F113">
-    <cfRule type="dataBar" priority="11">
+  <conditionalFormatting sqref="F86:F100">
+    <cfRule type="dataBar" priority="10">
       <dataBar minLength="5" maxLength="90" showValue="1">
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5075,9 +4759,9 @@
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="66" t="inlineStr">
-        <is>
-          <t>除權息 4 檔 (1203 / 3661 / 7780 ...)</t>
+      <c r="C25" s="68" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -28138,7 +27822,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-03 22:54 TW | 1/1 success | 來源: 富邦1/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-04 01:22 TW | 1/1 success | 來源: 富邦1/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-04 02:18
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -2034,7 +2034,7 @@
         <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>39193</v>
+        <v>38483</v>
       </c>
     </row>
     <row r="21">
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="G32" s="257" t="n">
-        <v>-199.54917</v>
+        <v>-199.32547</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="G33" s="259" t="n">
-        <v>0.1706536496408914</v>
+        <v>0.170329424857283</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.7%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2677,11 +2677,11 @@
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>881453</v>
+        <v>870535</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -3220,7 +3220,7 @@
         </is>
       </c>
       <c r="C66" s="33" t="n">
-        <v>819686</v>
+        <v>809114</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>40121</v>
       </c>
       <c r="J66" s="213" t="n">
-        <v>0.199874464124067</v>
+        <v>0.2024861026965552</v>
       </c>
     </row>
     <row r="67">
@@ -4782,7 +4782,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="70" t="inlineStr">
         <is>
-          <t>-200 億 淨買</t>
+          <t>-199 億 淨買</t>
         </is>
       </c>
     </row>
@@ -17254,7 +17254,7 @@
         </is>
       </c>
       <c r="E189" s="133" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F189" s="133" t="n">
         <v>4</v>
@@ -17269,7 +17269,7 @@
         <v>36163</v>
       </c>
       <c r="J189" s="134" t="n">
-        <v>1349.28</v>
+        <v>1344.34</v>
       </c>
       <c r="K189" s="134" t="n">
         <v>1342.5</v>
@@ -17289,10 +17289,10 @@
         </is>
       </c>
       <c r="E190" s="133" t="n">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F190" s="133" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G190" s="133" t="n">
         <v>6900</v>
@@ -17304,10 +17304,10 @@
         <v>5108</v>
       </c>
       <c r="J190" s="134" t="n">
-        <v>413.15</v>
+        <v>425.9</v>
       </c>
       <c r="K190" s="134" t="n">
-        <v>416.79</v>
+        <v>448.05</v>
       </c>
       <c r="L190" s="237">
         <f>F190*(K190-J190)</f>
@@ -17324,7 +17324,7 @@
         </is>
       </c>
       <c r="E191" s="133" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F191" s="133" t="n">
         <v>15</v>
@@ -17339,7 +17339,7 @@
         <v>5017</v>
       </c>
       <c r="J191" s="134" t="n">
-        <v>470.85</v>
+        <v>478.7</v>
       </c>
       <c r="K191" s="134" t="n">
         <v>484.53</v>
@@ -17394,10 +17394,10 @@
         </is>
       </c>
       <c r="E193" s="133" t="n">
-        <v>195</v>
+        <v>101</v>
       </c>
       <c r="F193" s="133" t="n">
-        <v>121</v>
+        <v>45</v>
       </c>
       <c r="G193" s="133" t="n">
         <v>4975</v>
@@ -17409,12 +17409,12 @@
         <v>2627</v>
       </c>
       <c r="J193" s="134" t="n">
-        <v>255.14</v>
+        <v>492.6</v>
       </c>
       <c r="K193" s="134" t="n">
-        <v>194.01</v>
-      </c>
-      <c r="L193" s="236">
+        <v>521.67</v>
+      </c>
+      <c r="L193" s="237">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -17429,10 +17429,10 @@
         </is>
       </c>
       <c r="E194" s="133" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F194" s="133" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G194" s="133" t="n">
         <v>4190</v>
@@ -17444,12 +17444,12 @@
         <v>3002</v>
       </c>
       <c r="J194" s="134" t="n">
-        <v>634.8200000000001</v>
+        <v>654.66</v>
       </c>
       <c r="K194" s="134" t="n">
-        <v>625</v>
-      </c>
-      <c r="L194" s="236">
+        <v>698.53</v>
+      </c>
+      <c r="L194" s="237">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -17464,10 +17464,10 @@
         </is>
       </c>
       <c r="E195" s="133" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F195" s="133" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G195" s="133" t="n">
         <v>3951</v>
@@ -17479,10 +17479,10 @@
         <v>2153</v>
       </c>
       <c r="J195" s="134" t="n">
-        <v>940.67</v>
+        <v>1067.78</v>
       </c>
       <c r="K195" s="134" t="n">
-        <v>899</v>
+        <v>1057.65</v>
       </c>
       <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
@@ -17565,29 +17565,29 @@
       <c r="C198" s="135" t="n"/>
       <c r="D198" s="132" t="inlineStr">
         <is>
-          <t>晶豪科(3006)</t>
+          <t>富喬(1815)</t>
         </is>
       </c>
       <c r="E198" s="133" t="n">
-        <v>111</v>
+        <v>237</v>
       </c>
       <c r="F198" s="133" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="G198" s="133" t="n">
-        <v>3075</v>
+        <v>2864</v>
       </c>
       <c r="H198" s="133" t="n">
-        <v>2493</v>
+        <v>441</v>
       </c>
       <c r="I198" s="133" t="n">
-        <v>582</v>
+        <v>2423</v>
       </c>
       <c r="J198" s="134" t="n">
-        <v>277</v>
+        <v>120.84</v>
       </c>
       <c r="K198" s="134" t="n">
-        <v>277</v>
+        <v>126</v>
       </c>
       <c r="L198" s="237">
         <f>F198*(K198-J198)</f>
@@ -27822,7 +27822,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-04 01:22 TW | 1/1 success | 來源: 富邦1/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-04 02:18 TW | 1/1 success | 來源: 富邦1/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-05 01:12
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="30">
+  <numFmts count="31">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -55,6 +55,7 @@
     <numFmt numFmtId="191" formatCode="+0&quot; 億 (昨-199/5d-122)&quot;;-0&quot; 億 (昨-199/5d-122)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="192" formatCode="0&quot; 檔 +36億 &quot;&quot;(昨14/5d13)&quot;"/>
     <numFmt numFmtId="193" formatCode="0.0%&quot; 市-444億 &quot;&quot;(昨17/5d18)&quot;"/>
+    <numFmt numFmtId="194" formatCode="0.0%&quot; 市-446億 &quot;&quot;(昨17/5d18)&quot;"/>
   </numFmts>
   <fonts count="55">
     <font>
@@ -643,7 +644,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="266">
+  <cellXfs count="267">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1268,6 +1269,9 @@
     <xf numFmtId="193" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="194" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2576,8 +2580,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G32" s="265" t="n">
-        <v>0.1701493816780536</v>
+      <c r="G32" s="266" t="n">
+        <v>0.1700160365736953</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -9516,7 +9520,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="101" t="inlineStr">
         <is>
-          <t>大牌分析師 近 96/96 交易日出手 4599 次 (649 檔), 風格分布: 隔日沖近似 34% / 當沖 14% / 留倉 52%, 漲停命中 3% (其中 🔒鎖漲停 2%), 前 5 大集中 19%, 長線部位 76% (100 檔), ⚠️ 處置股部位 7% (20 檔), 📦 連續囤貨 52 檔 (最長 13 天 009816, 3 檔仍 active)。 主軸: 📈 長線持有/高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 96/96 交易日出手 4599 次 (649 檔), 風格分布: 隔日沖近似 34% / 當沖 14% / 留倉 52%, 漲停命中 3% (其中 🔒鎖漲停 2%), 前 5 大集中 19%, 長線部位 76% (100 檔), ⚠️ 處置股部位 9% (20 檔), 📦 連續囤貨 52 檔 (最長 13 天 009816, 3 檔仍 active)。 主軸: 📈 長線持有/高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>
@@ -28039,7 +28043,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="204" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-09-04 21:38 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-09-05 01:12 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>